<commit_message>
Add 30 angel network / seed fund investor records
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F19FGkn59tio4UCKXfsejn
</commit_message>
<xml_diff>
--- a/finance/Vytalix_Financial_Model_3yr.xlsx
+++ b/finance/Vytalix_Financial_Model_3yr.xlsx
@@ -990,7 +990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -1006,7 +1006,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Status: SCENARIO MODEL v1, built 7 September 2026 by finance/build_model.py. GBP. UK-domiciled entity (to be incorporated — TO VALIDATE).</t>
+          <t>Status: SCENARIO MODEL v1.1, built 7 September 2026 and revised 8 September 2026 by finance/build_model.py. GBP. UK-domiciled entity (to be incorporated — TO VALIDATE).</t>
         </is>
       </c>
     </row>
@@ -1144,33 +1144,85 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>SOURCES CITED (retrieved 7 Sept 2026 via web search; verify on gov.uk before external use)</t>
+          <t>CHANGE LOG — 8 SEPTEMBER 2026 (sanity-check revision; see notes on each Assumptions row)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Employer NI 15%, secondary threshold £5,000, Employment Allowance £10,500 (2026/27): https://www.moorepay.co.uk/payroll-hr-rates/tax-and-national-insurance-changes/ ; https://employerscalculator.co.uk/guides/employer-ni-rates-2026-27</t>
+          <t>1. Opening cash £25k/£35k/£50k (was £10k/£20k/£30k) and founder draw from month 4/3/3 (was 4/2/1): cash was negative in months 2–5 of every scenario before the pre-seed landed.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Auto-enrolment 3% employer minimum on qualifying earnings £6,240–£50,270 (2026/27): https://www.moorepay.co.uk/payroll-hr-rates/automatic-enrolment/</t>
+          <t>2. Conservative no longer hires Developer 1 (month 19 → not hired): with a £250k pre-seed, cash went negative at month 31. Conservative now ends month 36 with ~£21k and ~2 months' runway — the honest 'services-only' outcome.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>SEIS: £250k company lifetime cap, £200k investor cap, gross assets &lt; £350k, &lt; 3 years trading, &lt; 25 employees: https://thecarry.co.uk/essentials/seis-and-eis-limits-and-thresholds-for-2026 ; https://www.gov.uk/government/statistics/enterprise-investment-scheme-and-seed-enterprise-investment-scheme-may-2026/enterprise-investment-scheme-and-seed-enterprise-investment-scheme-2026</t>
+          <t>3. Base Y3 and High-growth Y2–Y3 operating costs raised (contractors, technology, marketing, compliance, travel, operations) so the seed is actually spent on scaling. Before: Base burned ~£20k/month after a £2m seed; High-growth was EBITDA-positive from month 2 with £11m unspent at month 36.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>4. Series A removed from the 36-month model (was £6m at month 32 in High-growth, raised while cash-generative). No scenario needs it for solvency within 36 months; it is a month 30–42 decision in 09_FUNDING_STRATEGY. The input rows remain for testing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>5. Added 'sustained break-even' (first month from which EBITDA stays positive to month 36) to P&amp;L, Funding requirement (row 20), Dashboard and Static summary — the previous 'first positive month' was a pre-salary blip (month 2–4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>6. Build order fix: the P&amp;L grant row and the Opening-cash row reference rows built later; the builder now runs a two-pass layout so every formula points at a real row. Formula-reference checker no longer flags string concatenations (&amp;Assumptions!D4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>SOURCES CITED (retrieved 7 Sept 2026 via web search; verify on gov.uk before external use)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Employer NI 15%, secondary threshold £5,000, Employment Allowance £10,500 (2026/27): https://www.moorepay.co.uk/payroll-hr-rates/tax-and-national-insurance-changes/ ; https://employerscalculator.co.uk/guides/employer-ni-rates-2026-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Auto-enrolment 3% employer minimum on qualifying earnings £6,240–£50,270 (2026/27): https://www.moorepay.co.uk/payroll-hr-rates/automatic-enrolment/</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>SEIS: £250k company lifetime cap, £200k investor cap, gross assets &lt; £350k, &lt; 3 years trading, &lt; 25 employees: https://thecarry.co.uk/essentials/seis-and-eis-limits-and-thresholds-for-2026 ; https://www.gov.uk/government/statistics/enterprise-investment-scheme-and-seed-enterprise-investment-scheme-may-2026/enterprise-investment-scheme-and-seed-enterprise-investment-scheme-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>EIS from 6 April 2026: £10m per 12 months (£20m knowledge-intensive), £24m lifetime (£40m KIC), gross assets £30m/£35m, investor £1m (£2m KIC): https://www.farrer.co.uk/news-and-insights/using-eis-and-seis-to-attract-investment-the-benefits-and-some-traps-to-avoid/ ; https://ct.me/content-hub/articles/eis-changes-from-april-2026-higher-investment-limits-for-innovative-companies/</t>
         </is>
@@ -1187,7 +1239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1451,19 +1503,19 @@
         </is>
       </c>
       <c r="B14" s="19">
-        <f>'P&amp;L'!AN34</f>
+        <f>'P&amp;L'!AN35</f>
         <v/>
       </c>
       <c r="C14" s="19">
-        <f>'P&amp;L'!AO34</f>
+        <f>'P&amp;L'!AO35</f>
         <v/>
       </c>
       <c r="D14" s="19">
-        <f>'P&amp;L'!AP34</f>
+        <f>'P&amp;L'!AP35</f>
         <v/>
       </c>
       <c r="E14" s="19">
-        <f>'P&amp;L'!AQ34</f>
+        <f>'P&amp;L'!AQ35</f>
         <v/>
       </c>
     </row>
@@ -1474,19 +1526,19 @@
         </is>
       </c>
       <c r="B15" s="19">
-        <f>'P&amp;L'!AN35</f>
+        <f>'P&amp;L'!AN36</f>
         <v/>
       </c>
       <c r="C15" s="19">
-        <f>'P&amp;L'!AO35</f>
+        <f>'P&amp;L'!AO36</f>
         <v/>
       </c>
       <c r="D15" s="19">
-        <f>'P&amp;L'!AP35</f>
+        <f>'P&amp;L'!AP36</f>
         <v/>
       </c>
       <c r="E15" s="19">
-        <f>'P&amp;L'!AQ35</f>
+        <f>'P&amp;L'!AQ36</f>
         <v/>
       </c>
     </row>
@@ -1625,32 +1677,43 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Minimum closing cash after funding</t>
-        </is>
-      </c>
-      <c r="B25" s="30">
-        <f>'Funding requirement'!B10</f>
+          <t>First month of sustained positive EBITDA</t>
+        </is>
+      </c>
+      <c r="B25" s="31">
+        <f>'Funding requirement'!B20</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Funded-through check</t>
-        </is>
-      </c>
-      <c r="B26" s="7">
-        <f>'Funding requirement'!B12</f>
+          <t>Minimum closing cash after funding</t>
+        </is>
+      </c>
+      <c r="B26" s="30">
+        <f>'Funding requirement'!B10</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>Funded-through check</t>
+        </is>
+      </c>
+      <c r="B27" s="7">
+        <f>'Funding requirement'!B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>Runway at month 36 (months)</t>
         </is>
       </c>
-      <c r="B27" s="32">
+      <c r="B28" s="32">
         <f>'Funding requirement'!B14</f>
         <v/>
       </c>
@@ -1805,13 +1868,13 @@
         </is>
       </c>
       <c r="B12" s="19" t="n">
-        <v>428166</v>
+        <v>1082925</v>
       </c>
       <c r="C12" s="19" t="n">
-        <v>408426</v>
+        <v>1063184</v>
       </c>
       <c r="D12" s="19" t="n">
-        <v>383382</v>
+        <v>1038140</v>
       </c>
     </row>
     <row r="13">
@@ -1821,13 +1884,13 @@
         </is>
       </c>
       <c r="B13" s="19" t="n">
-        <v>428166</v>
+        <v>1082925</v>
       </c>
       <c r="C13" s="19" t="n">
-        <v>403277</v>
+        <v>1058035</v>
       </c>
       <c r="D13" s="19" t="n">
-        <v>371699</v>
+        <v>1026457</v>
       </c>
     </row>
     <row r="14">
@@ -1837,13 +1900,13 @@
         </is>
       </c>
       <c r="B14" s="19" t="n">
-        <v>428166</v>
+        <v>1082925</v>
       </c>
       <c r="C14" s="19" t="n">
-        <v>398127</v>
+        <v>1052885</v>
       </c>
       <c r="D14" s="19" t="n">
-        <v>360016</v>
+        <v>1014774</v>
       </c>
     </row>
     <row r="16">
@@ -1881,13 +1944,13 @@
         </is>
       </c>
       <c r="B18" s="19" t="n">
-        <v>-387333</v>
+        <v>-1057091</v>
       </c>
       <c r="C18" s="19" t="n">
-        <v>-367593</v>
+        <v>-1037351</v>
       </c>
       <c r="D18" s="19" t="n">
-        <v>-342548</v>
+        <v>-1012306</v>
       </c>
     </row>
     <row r="19">
@@ -1897,13 +1960,13 @@
         </is>
       </c>
       <c r="B19" s="19" t="n">
-        <v>-387333</v>
+        <v>-1057091</v>
       </c>
       <c r="C19" s="19" t="n">
-        <v>-362443</v>
+        <v>-1032201</v>
       </c>
       <c r="D19" s="19" t="n">
-        <v>-330865</v>
+        <v>-1000623</v>
       </c>
     </row>
     <row r="20">
@@ -1913,13 +1976,13 @@
         </is>
       </c>
       <c r="B20" s="19" t="n">
-        <v>-387333</v>
+        <v>-1057091</v>
       </c>
       <c r="C20" s="19" t="n">
-        <v>-357294</v>
+        <v>-1027052</v>
       </c>
       <c r="D20" s="19" t="n">
-        <v>-319182</v>
+        <v>-988940</v>
       </c>
     </row>
     <row r="22">
@@ -1985,16 +2048,16 @@
         <v>1474289</v>
       </c>
       <c r="D24" s="19" t="n">
-        <v>-362443</v>
+        <v>-1032201</v>
       </c>
       <c r="E24" s="19" t="n">
-        <v>403277</v>
+        <v>1058035</v>
       </c>
       <c r="F24" t="n">
         <v>4</v>
       </c>
       <c r="G24" s="19" t="n">
-        <v>2071723</v>
+        <v>1416965</v>
       </c>
     </row>
     <row r="25">
@@ -2010,16 +2073,16 @@
         <v>1432289</v>
       </c>
       <c r="D25" s="19" t="n">
-        <v>-389218</v>
+        <v>-1058976</v>
       </c>
       <c r="E25" s="19" t="n">
-        <v>428052</v>
+        <v>1082810</v>
       </c>
       <c r="F25" t="n">
         <v>4</v>
       </c>
       <c r="G25" s="19" t="n">
-        <v>2046948</v>
+        <v>1392190</v>
       </c>
     </row>
     <row r="26">
@@ -2035,16 +2098,16 @@
         <v>1396289</v>
       </c>
       <c r="D26" s="19" t="n">
-        <v>-412168</v>
+        <v>-1081926</v>
       </c>
       <c r="E26" s="19" t="n">
-        <v>449002</v>
+        <v>1103760</v>
       </c>
       <c r="F26" t="n">
         <v>4</v>
       </c>
       <c r="G26" s="19" t="n">
-        <v>2025998</v>
+        <v>1371240</v>
       </c>
     </row>
     <row r="27">
@@ -2060,16 +2123,16 @@
         <v>1342289</v>
       </c>
       <c r="D27" s="19" t="n">
-        <v>-446593</v>
+        <v>-1116351</v>
       </c>
       <c r="E27" s="19" t="n">
-        <v>479427</v>
+        <v>1134185</v>
       </c>
       <c r="F27" t="n">
         <v>4</v>
       </c>
       <c r="G27" s="19" t="n">
-        <v>1995573</v>
+        <v>1340815</v>
       </c>
     </row>
     <row r="29">
@@ -2135,16 +2198,16 @@
         <v>5249714</v>
       </c>
       <c r="D31" s="19" t="n">
-        <v>1644390</v>
+        <v>113985</v>
       </c>
       <c r="E31" s="19" t="n">
-        <v>36337</v>
+        <v>144705</v>
       </c>
       <c r="F31" t="n">
         <v>2</v>
       </c>
       <c r="G31" s="19" t="n">
-        <v>11350390</v>
+        <v>3839985</v>
       </c>
     </row>
     <row r="32">
@@ -2160,16 +2223,16 @@
         <v>4949714</v>
       </c>
       <c r="D32" s="19" t="n">
-        <v>1408140</v>
+        <v>-122265</v>
       </c>
       <c r="E32" s="19" t="n">
-        <v>36337</v>
+        <v>326751</v>
       </c>
       <c r="F32" t="n">
         <v>2</v>
       </c>
       <c r="G32" s="19" t="n">
-        <v>11126140</v>
+        <v>3615735</v>
       </c>
     </row>
     <row r="33">
@@ -2185,16 +2248,16 @@
         <v>4685714</v>
       </c>
       <c r="D33" s="19" t="n">
-        <v>1200240</v>
+        <v>-330165</v>
       </c>
       <c r="E33" s="19" t="n">
-        <v>36337</v>
+        <v>495471</v>
       </c>
       <c r="F33" t="n">
         <v>2</v>
       </c>
       <c r="G33" s="19" t="n">
-        <v>10930240</v>
+        <v>3419835</v>
       </c>
     </row>
     <row r="34">
@@ -2210,16 +2273,16 @@
         <v>4265714</v>
       </c>
       <c r="D34" s="19" t="n">
-        <v>869490</v>
+        <v>-660915</v>
       </c>
       <c r="E34" s="19" t="n">
-        <v>36337</v>
+        <v>786915</v>
       </c>
       <c r="F34" t="n">
         <v>2</v>
       </c>
       <c r="G34" s="19" t="n">
-        <v>10623490</v>
+        <v>3113085</v>
       </c>
     </row>
     <row r="36">
@@ -2285,16 +2348,16 @@
         <v>412514</v>
       </c>
       <c r="D38" s="19" t="n">
-        <v>-326637</v>
+        <v>-239543</v>
       </c>
       <c r="E38" s="19" t="n">
-        <v>330967</v>
+        <v>228872</v>
       </c>
       <c r="F38" t="n">
         <v>3</v>
       </c>
       <c r="G38" s="19" t="n">
-        <v>-80967</v>
+        <v>21128</v>
       </c>
     </row>
     <row r="39">
@@ -2310,16 +2373,16 @@
         <v>409064</v>
       </c>
       <c r="D39" s="19" t="n">
-        <v>-327987</v>
+        <v>-240893</v>
       </c>
       <c r="E39" s="19" t="n">
-        <v>332029</v>
+        <v>229935</v>
       </c>
       <c r="F39" t="n">
         <v>3</v>
       </c>
       <c r="G39" s="19" t="n">
-        <v>-82029</v>
+        <v>20065</v>
       </c>
     </row>
     <row r="40">
@@ -2335,16 +2398,16 @@
         <v>406477</v>
       </c>
       <c r="D40" s="19" t="n">
-        <v>-329000</v>
+        <v>-241906</v>
       </c>
       <c r="E40" s="19" t="n">
-        <v>332754</v>
+        <v>230660</v>
       </c>
       <c r="F40" t="n">
         <v>3</v>
       </c>
       <c r="G40" s="19" t="n">
-        <v>-82754</v>
+        <v>19340</v>
       </c>
     </row>
     <row r="41">
@@ -2360,22 +2423,22 @@
         <v>404369</v>
       </c>
       <c r="D41" s="19" t="n">
-        <v>-329825</v>
+        <v>-242731</v>
       </c>
       <c r="E41" s="19" t="n">
-        <v>332908</v>
+        <v>230814</v>
       </c>
       <c r="F41" t="n">
         <v>3</v>
       </c>
       <c r="G41" s="19" t="n">
-        <v>-82908</v>
+        <v>19186</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>Table — Base scenario one-at-a-time flex (Base 3-yr revenue £1,474,289; 3-yr EBITDA £-362,443; peak need £403,277)</t>
+          <t>Table — Base scenario one-at-a-time flex (Base 3-yr revenue £1,474,289; 3-yr EBITDA £-1,032,201; peak need £1,058,035)</t>
         </is>
       </c>
       <c r="B43" s="10" t="n"/>
@@ -2724,7 +2787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F89"/>
+  <dimension ref="A1:F92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -2930,13 +2993,13 @@
         <v>31157.1</v>
       </c>
       <c r="C13" s="19" t="n">
-        <v>129645.1</v>
+        <v>100613.7</v>
       </c>
       <c r="D13" s="19" t="n">
-        <v>158676.5</v>
+        <v>100613.7</v>
       </c>
       <c r="E13" s="19" t="n">
-        <v>319478.7</v>
+        <v>232384.5</v>
       </c>
     </row>
     <row r="14">
@@ -2949,13 +3012,13 @@
         <v>84037.10000000001</v>
       </c>
       <c r="C14" s="19" t="n">
-        <v>217845.1</v>
+        <v>188813.7</v>
       </c>
       <c r="D14" s="19" t="n">
-        <v>340476.5</v>
+        <v>282413.7</v>
       </c>
       <c r="E14" s="19" t="n">
-        <v>642358.7</v>
+        <v>555264.5</v>
       </c>
     </row>
     <row r="15">
@@ -2968,13 +3031,13 @@
         <v>-21659.69</v>
       </c>
       <c r="C15" s="19" t="n">
-        <v>-106197.09</v>
+        <v>-77165.69</v>
       </c>
       <c r="D15" s="19" t="n">
-        <v>-198780.7</v>
+        <v>-140717.9</v>
       </c>
       <c r="E15" s="19" t="n">
-        <v>-326637.48</v>
+        <v>-239543.28</v>
       </c>
     </row>
     <row r="16">
@@ -3006,13 +3069,13 @@
         <v>-21659.69</v>
       </c>
       <c r="C17" s="19" t="n">
-        <v>-106197.09</v>
+        <v>-77165.69</v>
       </c>
       <c r="D17" s="19" t="n">
-        <v>-198780.7</v>
+        <v>-140717.9</v>
       </c>
       <c r="E17" s="19" t="n">
-        <v>-326637.48</v>
+        <v>-239543.28</v>
       </c>
     </row>
     <row r="18">
@@ -3025,13 +3088,13 @@
         <v>-29048.49</v>
       </c>
       <c r="C18" s="19" t="n">
-        <v>-110680.42</v>
+        <v>-81649.02</v>
       </c>
       <c r="D18" s="19" t="n">
-        <v>-201237.73</v>
+        <v>-143174.93</v>
       </c>
       <c r="E18" s="19" t="n">
-        <v>-340966.64</v>
+        <v>-253872.44</v>
       </c>
     </row>
     <row r="19">
@@ -3041,16 +3104,16 @@
         </is>
       </c>
       <c r="B19" s="19" t="n">
-        <v>230951.51</v>
+        <v>245951.51</v>
       </c>
       <c r="C19" s="19" t="n">
-        <v>120271.09</v>
+        <v>164302.49</v>
       </c>
       <c r="D19" s="19" t="n">
-        <v>-80966.64</v>
+        <v>21127.56</v>
       </c>
       <c r="E19" s="19" t="n">
-        <v>-80966.64</v>
+        <v>21127.56</v>
       </c>
     </row>
     <row r="20">
@@ -3063,13 +3126,13 @@
         <v>1</v>
       </c>
       <c r="C20" s="27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D20" s="27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E20" s="27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
@@ -3098,7 +3161,7 @@
         </is>
       </c>
       <c r="B22" s="30" t="n">
-        <v>330966.64</v>
+        <v>228872.44</v>
       </c>
     </row>
     <row r="23">
@@ -3114,7 +3177,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>First month with positive EBITDA</t>
+          <t>First month with positive EBITDA (may be a blip)</t>
         </is>
       </c>
       <c r="B24" s="31" t="n">
@@ -3124,7 +3187,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>First month cumulative result positive</t>
+          <t>First month of SUSTAINED positive EBITDA (break-even)</t>
         </is>
       </c>
       <c r="B25" s="31" t="inlineStr">
@@ -3136,946 +3199,982 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Minimum closing cash after funding</t>
-        </is>
-      </c>
-      <c r="B26" s="30" t="n">
-        <v>-80966.64</v>
+          <t>First month cumulative result positive</t>
+        </is>
+      </c>
+      <c r="B26" s="31" t="inlineStr">
+        <is>
+          <t>Not reached in 36 months</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Month of minimum closing cash</t>
-        </is>
-      </c>
-      <c r="B27" s="31" t="n">
-        <v>36</v>
+          <t>Minimum closing cash after funding</t>
+        </is>
+      </c>
+      <c r="B27" s="30" t="n">
+        <v>4726.19</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Closing cash month 36</t>
-        </is>
-      </c>
-      <c r="B28" s="30" t="n">
-        <v>-80966.64</v>
+          <t>Month of minimum closing cash</t>
+        </is>
+      </c>
+      <c r="B28" s="31" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Equity raised in model</t>
+          <t>Closing cash month 36</t>
         </is>
       </c>
       <c r="B29" s="30" t="n">
-        <v>250000</v>
+        <v>21127.56</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Grants in model</t>
+          <t>Equity raised in model</t>
         </is>
       </c>
       <c r="B30" s="30" t="n">
-        <v>0</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>Grants in model</t>
+        </is>
+      </c>
+      <c r="B31" s="30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>Runway at month 36 (months)</t>
         </is>
       </c>
-      <c r="B31" s="32" t="n">
-        <v>-4.99</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="9" t="inlineStr">
+      <c r="B32" s="32" t="n">
+        <v>1.85</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
         <is>
           <t>Base scenario — annual P&amp;L and cash</t>
         </is>
       </c>
-      <c r="B33" s="10" t="n"/>
-      <c r="C33" s="10" t="n"/>
-      <c r="D33" s="10" t="n"/>
-      <c r="E33" s="10" t="n"/>
-      <c r="F33" s="10" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="7" t="inlineStr">
+      <c r="B34" s="10" t="n"/>
+      <c r="C34" s="10" t="n"/>
+      <c r="D34" s="10" t="n"/>
+      <c r="E34" s="10" t="n"/>
+      <c r="F34" s="10" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
         <is>
           <t>Line</t>
         </is>
       </c>
-      <c r="B34" s="7" t="inlineStr">
+      <c r="B35" s="7" t="inlineStr">
         <is>
           <t>FY2027</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
+      <c r="C35" s="7" t="inlineStr">
         <is>
           <t>FY2028</t>
         </is>
       </c>
-      <c r="D34" s="7" t="inlineStr">
+      <c r="D35" s="7" t="inlineStr">
         <is>
           <t>FY2029</t>
         </is>
       </c>
-      <c r="E34" s="7" t="inlineStr">
+      <c r="E35" s="7" t="inlineStr">
         <is>
           <t>3-year</t>
         </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="22" t="inlineStr">
-        <is>
-          <t>Advisory</t>
-        </is>
-      </c>
-      <c r="B35" s="19" t="n">
-        <v>69748.03</v>
-      </c>
-      <c r="C35" s="19" t="n">
-        <v>150000</v>
-      </c>
-      <c r="D35" s="19" t="n">
-        <v>204000</v>
-      </c>
-      <c r="E35" s="19" t="n">
-        <v>423748.03</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="22" t="inlineStr">
         <is>
-          <t>Consulting</t>
+          <t>Advisory</t>
         </is>
       </c>
       <c r="B36" s="19" t="n">
-        <v>83333.33</v>
+        <v>69748.03</v>
       </c>
       <c r="C36" s="19" t="n">
-        <v>160000</v>
+        <v>150000</v>
       </c>
       <c r="D36" s="19" t="n">
-        <v>200000</v>
+        <v>204000</v>
       </c>
       <c r="E36" s="19" t="n">
-        <v>443333.33</v>
+        <v>423748.03</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="22" t="inlineStr">
         <is>
-          <t>E-learning</t>
+          <t>Consulting</t>
         </is>
       </c>
       <c r="B37" s="19" t="n">
-        <v>12930.38</v>
+        <v>83333.33</v>
       </c>
       <c r="C37" s="19" t="n">
-        <v>73042.10000000001</v>
+        <v>160000</v>
       </c>
       <c r="D37" s="19" t="n">
-        <v>134235.27</v>
+        <v>200000</v>
       </c>
       <c r="E37" s="19" t="n">
-        <v>220207.75</v>
+        <v>443333.33</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="22" t="inlineStr">
         <is>
+          <t>E-learning</t>
+        </is>
+      </c>
+      <c r="B38" s="19" t="n">
+        <v>12930.38</v>
+      </c>
+      <c r="C38" s="19" t="n">
+        <v>73042.10000000001</v>
+      </c>
+      <c r="D38" s="19" t="n">
+        <v>134235.27</v>
+      </c>
+      <c r="E38" s="19" t="n">
+        <v>220207.75</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="22" t="inlineStr">
+        <is>
           <t>MaternaLink (in development)</t>
         </is>
       </c>
-      <c r="B38" s="19" t="n">
+      <c r="B39" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="C38" s="19" t="n">
+      <c r="C39" s="19" t="n">
         <v>105000</v>
       </c>
-      <c r="D38" s="19" t="n">
+      <c r="D39" s="19" t="n">
         <v>282000</v>
       </c>
-      <c r="E38" s="19" t="n">
+      <c r="E39" s="19" t="n">
         <v>387000</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="7" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
         <is>
           <t>TOTAL REVENUE</t>
         </is>
       </c>
-      <c r="B39" s="19" t="n">
+      <c r="B40" s="19" t="n">
         <v>166011.74</v>
       </c>
-      <c r="C39" s="19" t="n">
+      <c r="C40" s="19" t="n">
         <v>488042.1</v>
       </c>
-      <c r="D39" s="19" t="n">
+      <c r="D40" s="19" t="n">
         <v>820235.27</v>
       </c>
-      <c r="E39" s="19" t="n">
+      <c r="E40" s="19" t="n">
         <v>1474289.11</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="22" t="inlineStr">
-        <is>
-          <t>Cost of sales</t>
-        </is>
-      </c>
-      <c r="B40" s="19" t="n">
-        <v>33339.49</v>
-      </c>
-      <c r="C40" s="19" t="n">
-        <v>114581.32</v>
-      </c>
-      <c r="D40" s="19" t="n">
-        <v>208485.29</v>
-      </c>
-      <c r="E40" s="19" t="n">
-        <v>356406.1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="22" t="inlineStr">
         <is>
-          <t>Gross profit</t>
+          <t>Cost of sales</t>
         </is>
       </c>
       <c r="B41" s="19" t="n">
-        <v>132672.25</v>
+        <v>33339.49</v>
       </c>
       <c r="C41" s="19" t="n">
-        <v>373460.79</v>
+        <v>114581.32</v>
       </c>
       <c r="D41" s="19" t="n">
-        <v>611749.98</v>
+        <v>208485.29</v>
       </c>
       <c r="E41" s="19" t="n">
-        <v>1117883.02</v>
+        <v>356406.1</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="22" t="inlineStr">
         <is>
-          <t>Employment cost</t>
+          <t>Gross profit</t>
         </is>
       </c>
       <c r="B42" s="19" t="n">
-        <v>99426.58</v>
+        <v>132672.25</v>
       </c>
       <c r="C42" s="19" t="n">
-        <v>290116.87</v>
+        <v>373460.79</v>
       </c>
       <c r="D42" s="19" t="n">
-        <v>485582.9</v>
+        <v>611749.98</v>
       </c>
       <c r="E42" s="19" t="n">
-        <v>875126.35</v>
+        <v>1117883.02</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="22" t="inlineStr">
         <is>
-          <t>Total operating expenses</t>
+          <t>Employment cost</t>
         </is>
       </c>
       <c r="B43" s="19" t="n">
-        <v>192826.57</v>
+        <v>94784.67999999999</v>
       </c>
       <c r="C43" s="19" t="n">
-        <v>458716.87</v>
+        <v>290116.87</v>
       </c>
       <c r="D43" s="19" t="n">
-        <v>828782.9</v>
+        <v>485582.9</v>
       </c>
       <c r="E43" s="19" t="n">
-        <v>1480326.35</v>
+        <v>870484.45</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="22" t="inlineStr">
         <is>
-          <t>EBITDA (before grants)</t>
+          <t>Total operating expenses</t>
         </is>
       </c>
       <c r="B44" s="19" t="n">
-        <v>-60154.32</v>
+        <v>188184.67</v>
       </c>
       <c r="C44" s="19" t="n">
-        <v>-85256.09</v>
+        <v>563116.88</v>
       </c>
       <c r="D44" s="19" t="n">
-        <v>-217032.92</v>
+        <v>1398782.9</v>
       </c>
       <c r="E44" s="19" t="n">
-        <v>-362443.33</v>
+        <v>2150084.45</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="22" t="inlineStr">
         <is>
-          <t>Grant income</t>
+          <t>EBITDA (before grants)</t>
         </is>
       </c>
       <c r="B45" s="19" t="n">
-        <v>0</v>
+        <v>-55512.42</v>
       </c>
       <c r="C45" s="19" t="n">
-        <v>75000</v>
+        <v>-189656.09</v>
       </c>
       <c r="D45" s="19" t="n">
-        <v>0</v>
+        <v>-787032.92</v>
       </c>
       <c r="E45" s="19" t="n">
-        <v>75000</v>
+        <v>-1032201.43</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="22" t="inlineStr">
         <is>
-          <t>Net result</t>
+          <t>Grant income</t>
         </is>
       </c>
       <c r="B46" s="19" t="n">
-        <v>-60154.32</v>
+        <v>0</v>
       </c>
       <c r="C46" s="19" t="n">
-        <v>-10256.09</v>
+        <v>75000</v>
       </c>
       <c r="D46" s="19" t="n">
-        <v>-217032.92</v>
+        <v>0</v>
       </c>
       <c r="E46" s="19" t="n">
-        <v>-287443.33</v>
+        <v>75000</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="22" t="inlineStr">
         <is>
-          <t>Net operating cash flow</t>
+          <t>Net result</t>
         </is>
       </c>
       <c r="B47" s="19" t="n">
-        <v>-75280.56</v>
+        <v>-55512.42</v>
       </c>
       <c r="C47" s="19" t="n">
-        <v>-113379.86</v>
+        <v>-114656.09</v>
       </c>
       <c r="D47" s="19" t="n">
-        <v>-234616.25</v>
+        <v>-787032.92</v>
       </c>
       <c r="E47" s="19" t="n">
-        <v>-423276.67</v>
+        <v>-957201.4300000001</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="22" t="inlineStr">
         <is>
-          <t>Closing cash (year end)</t>
+          <t>Net operating cash flow</t>
         </is>
       </c>
       <c r="B48" s="19" t="n">
-        <v>344719.44</v>
+        <v>-70638.66</v>
       </c>
       <c r="C48" s="19" t="n">
-        <v>2306339.59</v>
+        <v>-217779.86</v>
       </c>
       <c r="D48" s="19" t="n">
-        <v>2071723.33</v>
+        <v>-804616.25</v>
       </c>
       <c r="E48" s="19" t="n">
-        <v>2071723.33</v>
+        <v>-1093034.77</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="22" t="inlineStr">
         <is>
+          <t>Closing cash (year end)</t>
+        </is>
+      </c>
+      <c r="B49" s="19" t="n">
+        <v>364361.34</v>
+      </c>
+      <c r="C49" s="19" t="n">
+        <v>2221581.49</v>
+      </c>
+      <c r="D49" s="19" t="n">
+        <v>1416965.23</v>
+      </c>
+      <c r="E49" s="19" t="n">
+        <v>1416965.23</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="22" t="inlineStr">
+        <is>
           <t>Headcount (year end)</t>
         </is>
       </c>
-      <c r="B49" s="27" t="n">
+      <c r="B50" s="27" t="n">
         <v>3</v>
       </c>
-      <c r="C49" s="27" t="n">
+      <c r="C50" s="27" t="n">
         <v>7</v>
       </c>
-      <c r="D49" s="27" t="n">
+      <c r="D50" s="27" t="n">
         <v>8</v>
       </c>
-      <c r="E49" s="27" t="n">
+      <c r="E50" s="27" t="n">
         <v>8</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Gross margin %</t>
-        </is>
-      </c>
-      <c r="B50" s="25" t="n">
-        <v>0.7991738996306268</v>
-      </c>
-      <c r="C50" s="25" t="n">
-        <v>0.7652224777855855</v>
-      </c>
-      <c r="D50" s="25" t="n">
-        <v>0.7458225733368081</v>
-      </c>
-      <c r="E50" s="25" t="n">
-        <v>0.7582522362333166</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Peak cash need before external funding</t>
-        </is>
-      </c>
-      <c r="B51" s="30" t="n">
-        <v>403276.67</v>
+          <t>Gross margin %</t>
+        </is>
+      </c>
+      <c r="B51" s="25" t="n">
+        <v>0.7991738996306268</v>
+      </c>
+      <c r="C51" s="25" t="n">
+        <v>0.7652224777855855</v>
+      </c>
+      <c r="D51" s="25" t="n">
+        <v>0.7458225733368081</v>
+      </c>
+      <c r="E51" s="25" t="n">
+        <v>0.7582522362333166</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Month of peak cash need</t>
-        </is>
-      </c>
-      <c r="B52" s="31" t="n">
-        <v>36</v>
+          <t>Peak cash need before external funding</t>
+        </is>
+      </c>
+      <c r="B52" s="30" t="n">
+        <v>1058034.77</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>First month with positive EBITDA</t>
+          <t>Month of peak cash need</t>
         </is>
       </c>
       <c r="B53" s="31" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>First month cumulative result positive</t>
+          <t>First month with positive EBITDA (may be a blip)</t>
         </is>
       </c>
       <c r="B54" s="31" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Minimum closing cash after funding</t>
-        </is>
-      </c>
-      <c r="B55" s="30" t="n">
-        <v>-13543.09</v>
+          <t>First month of SUSTAINED positive EBITDA (break-even)</t>
+        </is>
+      </c>
+      <c r="B55" s="31" t="inlineStr">
+        <is>
+          <t>Not reached in 36 months</t>
+        </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Month of minimum closing cash</t>
-        </is>
-      </c>
-      <c r="B56" s="31" t="n">
-        <v>3</v>
+          <t>First month cumulative result positive</t>
+        </is>
+      </c>
+      <c r="B56" s="31" t="inlineStr">
+        <is>
+          <t>Not reached in 36 months</t>
+        </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Closing cash month 36</t>
+          <t>Minimum closing cash after funding</t>
         </is>
       </c>
       <c r="B57" s="30" t="n">
-        <v>2071723.33</v>
+        <v>6098.81</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Equity raised in model</t>
-        </is>
-      </c>
-      <c r="B58" s="30" t="n">
-        <v>2400000</v>
+          <t>Month of minimum closing cash</t>
+        </is>
+      </c>
+      <c r="B58" s="31" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Grants in model</t>
+          <t>Closing cash month 36</t>
         </is>
       </c>
       <c r="B59" s="30" t="n">
-        <v>75000</v>
+        <v>1416965.23</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
+          <t>Equity raised in model</t>
+        </is>
+      </c>
+      <c r="B60" s="30" t="n">
+        <v>2400000</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Grants in model</t>
+        </is>
+      </c>
+      <c r="B61" s="30" t="n">
+        <v>75000</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
           <t>Runway at month 36 (months)</t>
         </is>
       </c>
-      <c r="B60" s="32" t="n">
-        <v>136.75</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="9" t="inlineStr">
+      <c r="B62" s="32" t="n">
+        <v>22.62</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="9" t="inlineStr">
         <is>
           <t>High-growth scenario — annual P&amp;L and cash</t>
         </is>
       </c>
-      <c r="B62" s="10" t="n"/>
-      <c r="C62" s="10" t="n"/>
-      <c r="D62" s="10" t="n"/>
-      <c r="E62" s="10" t="n"/>
-      <c r="F62" s="10" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="7" t="inlineStr">
+      <c r="B64" s="10" t="n"/>
+      <c r="C64" s="10" t="n"/>
+      <c r="D64" s="10" t="n"/>
+      <c r="E64" s="10" t="n"/>
+      <c r="F64" s="10" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="7" t="inlineStr">
         <is>
           <t>Line</t>
         </is>
       </c>
-      <c r="B63" s="7" t="inlineStr">
+      <c r="B65" s="7" t="inlineStr">
         <is>
           <t>FY2027</t>
         </is>
       </c>
-      <c r="C63" s="7" t="inlineStr">
+      <c r="C65" s="7" t="inlineStr">
         <is>
           <t>FY2028</t>
         </is>
       </c>
-      <c r="D63" s="7" t="inlineStr">
+      <c r="D65" s="7" t="inlineStr">
         <is>
           <t>FY2029</t>
         </is>
       </c>
-      <c r="E63" s="7" t="inlineStr">
+      <c r="E65" s="7" t="inlineStr">
         <is>
           <t>3-year</t>
         </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="22" t="inlineStr">
-        <is>
-          <t>Advisory</t>
-        </is>
-      </c>
-      <c r="B64" s="19" t="n">
-        <v>161567</v>
-      </c>
-      <c r="C64" s="19" t="n">
-        <v>300000</v>
-      </c>
-      <c r="D64" s="19" t="n">
-        <v>300000</v>
-      </c>
-      <c r="E64" s="19" t="n">
-        <v>761567</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="22" t="inlineStr">
-        <is>
-          <t>Consulting</t>
-        </is>
-      </c>
-      <c r="B65" s="19" t="n">
-        <v>210000</v>
-      </c>
-      <c r="C65" s="19" t="n">
-        <v>420000</v>
-      </c>
-      <c r="D65" s="19" t="n">
-        <v>540000</v>
-      </c>
-      <c r="E65" s="19" t="n">
-        <v>1170000</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="22" t="inlineStr">
         <is>
-          <t>E-learning</t>
+          <t>Advisory</t>
         </is>
       </c>
       <c r="B66" s="19" t="n">
-        <v>68879.62</v>
+        <v>161567</v>
       </c>
       <c r="C66" s="19" t="n">
-        <v>295611.68</v>
+        <v>300000</v>
       </c>
       <c r="D66" s="19" t="n">
-        <v>652155.78</v>
+        <v>300000</v>
       </c>
       <c r="E66" s="19" t="n">
-        <v>1016647.08</v>
+        <v>761567</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="22" t="inlineStr">
         <is>
-          <t>MaternaLink (in development)</t>
+          <t>Consulting</t>
         </is>
       </c>
       <c r="B67" s="19" t="n">
-        <v>37500</v>
+        <v>210000</v>
       </c>
       <c r="C67" s="19" t="n">
-        <v>680000</v>
+        <v>420000</v>
       </c>
       <c r="D67" s="19" t="n">
-        <v>1584000</v>
+        <v>540000</v>
       </c>
       <c r="E67" s="19" t="n">
-        <v>2301500</v>
+        <v>1170000</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="7" t="inlineStr">
-        <is>
-          <t>TOTAL REVENUE</t>
+      <c r="A68" s="22" t="inlineStr">
+        <is>
+          <t>E-learning</t>
         </is>
       </c>
       <c r="B68" s="19" t="n">
-        <v>477946.62</v>
+        <v>68879.62</v>
       </c>
       <c r="C68" s="19" t="n">
-        <v>1695611.68</v>
+        <v>295611.68</v>
       </c>
       <c r="D68" s="19" t="n">
-        <v>3076155.78</v>
+        <v>652155.78</v>
       </c>
       <c r="E68" s="19" t="n">
-        <v>5249714.08</v>
+        <v>1016647.08</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="22" t="inlineStr">
         <is>
-          <t>Cost of sales</t>
+          <t>MaternaLink (in development)</t>
         </is>
       </c>
       <c r="B69" s="19" t="n">
-        <v>123181.03</v>
+        <v>37500</v>
       </c>
       <c r="C69" s="19" t="n">
-        <v>438591.75</v>
+        <v>680000</v>
       </c>
       <c r="D69" s="19" t="n">
-        <v>794423.37</v>
+        <v>1584000</v>
       </c>
       <c r="E69" s="19" t="n">
-        <v>1356196.14</v>
+        <v>2301500</v>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="22" t="inlineStr">
-        <is>
-          <t>Gross profit</t>
+      <c r="A70" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL REVENUE</t>
         </is>
       </c>
       <c r="B70" s="19" t="n">
-        <v>354765.59</v>
+        <v>477946.62</v>
       </c>
       <c r="C70" s="19" t="n">
-        <v>1257019.92</v>
+        <v>1695611.68</v>
       </c>
       <c r="D70" s="19" t="n">
-        <v>2281732.42</v>
+        <v>3076155.78</v>
       </c>
       <c r="E70" s="19" t="n">
-        <v>3893517.93</v>
+        <v>5249714.08</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="22" t="inlineStr">
         <is>
-          <t>Employment cost</t>
+          <t>Cost of sales</t>
         </is>
       </c>
       <c r="B71" s="19" t="n">
-        <v>202227.62</v>
+        <v>123181.03</v>
       </c>
       <c r="C71" s="19" t="n">
-        <v>545607.85</v>
+        <v>438591.75</v>
       </c>
       <c r="D71" s="19" t="n">
-        <v>655692.8</v>
+        <v>794423.37</v>
       </c>
       <c r="E71" s="19" t="n">
-        <v>1403528.27</v>
+        <v>1356196.14</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="22" t="inlineStr">
         <is>
-          <t>Total operating expenses</t>
+          <t>Gross profit</t>
         </is>
       </c>
       <c r="B72" s="19" t="n">
-        <v>342227.62</v>
+        <v>354765.59</v>
       </c>
       <c r="C72" s="19" t="n">
-        <v>773607.85</v>
+        <v>1257019.92</v>
       </c>
       <c r="D72" s="19" t="n">
-        <v>1133292.8</v>
+        <v>2281732.42</v>
       </c>
       <c r="E72" s="19" t="n">
-        <v>2249128.28</v>
+        <v>3893517.93</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="22" t="inlineStr">
         <is>
-          <t>EBITDA (before grants)</t>
+          <t>Employment cost</t>
         </is>
       </c>
       <c r="B73" s="19" t="n">
-        <v>12537.97</v>
+        <v>190632.47</v>
       </c>
       <c r="C73" s="19" t="n">
-        <v>483412.07</v>
+        <v>545607.85</v>
       </c>
       <c r="D73" s="19" t="n">
-        <v>1148439.62</v>
+        <v>655692.8</v>
       </c>
       <c r="E73" s="19" t="n">
-        <v>1644389.66</v>
+        <v>1391933.12</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="22" t="inlineStr">
         <is>
-          <t>Grant income</t>
+          <t>Total operating expenses</t>
         </is>
       </c>
       <c r="B74" s="19" t="n">
-        <v>150000</v>
+        <v>330632.47</v>
       </c>
       <c r="C74" s="19" t="n">
-        <v>250000</v>
+        <v>1175607.85</v>
       </c>
       <c r="D74" s="19" t="n">
-        <v>0</v>
+        <v>2273292.8</v>
       </c>
       <c r="E74" s="19" t="n">
-        <v>400000</v>
+        <v>3779533.12</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="22" t="inlineStr">
         <is>
-          <t>Net result</t>
+          <t>EBITDA (before grants)</t>
         </is>
       </c>
       <c r="B75" s="19" t="n">
-        <v>162537.97</v>
+        <v>24133.12</v>
       </c>
       <c r="C75" s="19" t="n">
-        <v>733412.0699999999</v>
+        <v>81412.07000000001</v>
       </c>
       <c r="D75" s="19" t="n">
-        <v>1148439.62</v>
+        <v>8439.620000000001</v>
       </c>
       <c r="E75" s="19" t="n">
-        <v>2044389.66</v>
+        <v>113984.81</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="22" t="inlineStr">
         <is>
-          <t>Net operating cash flow</t>
+          <t>Grant income</t>
         </is>
       </c>
       <c r="B76" s="19" t="n">
-        <v>-42118.73</v>
+        <v>150000</v>
       </c>
       <c r="C76" s="19" t="n">
-        <v>397068.77</v>
+        <v>250000</v>
       </c>
       <c r="D76" s="19" t="n">
-        <v>1065439.62</v>
+        <v>0</v>
       </c>
       <c r="E76" s="19" t="n">
-        <v>1420389.66</v>
+        <v>400000</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="22" t="inlineStr">
         <is>
-          <t>Closing cash (year end)</t>
+          <t>Net result</t>
         </is>
       </c>
       <c r="B77" s="19" t="n">
-        <v>637881.27</v>
+        <v>174133.12</v>
       </c>
       <c r="C77" s="19" t="n">
-        <v>4284950.04</v>
+        <v>331412.07</v>
       </c>
       <c r="D77" s="19" t="n">
-        <v>11350389.66</v>
+        <v>8439.620000000001</v>
       </c>
       <c r="E77" s="19" t="n">
-        <v>11350389.66</v>
+        <v>513984.81</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="22" t="inlineStr">
         <is>
+          <t>Net operating cash flow</t>
+        </is>
+      </c>
+      <c r="B78" s="19" t="n">
+        <v>-30523.58</v>
+      </c>
+      <c r="C78" s="19" t="n">
+        <v>-4931.23</v>
+      </c>
+      <c r="D78" s="19" t="n">
+        <v>-74560.38</v>
+      </c>
+      <c r="E78" s="19" t="n">
+        <v>-110015.19</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="22" t="inlineStr">
+        <is>
+          <t>Closing cash (year end)</t>
+        </is>
+      </c>
+      <c r="B79" s="19" t="n">
+        <v>669476.42</v>
+      </c>
+      <c r="C79" s="19" t="n">
+        <v>3914545.19</v>
+      </c>
+      <c r="D79" s="19" t="n">
+        <v>3839984.81</v>
+      </c>
+      <c r="E79" s="19" t="n">
+        <v>3839984.81</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="22" t="inlineStr">
+        <is>
           <t>Headcount (year end)</t>
         </is>
       </c>
-      <c r="B78" s="27" t="n">
+      <c r="B80" s="27" t="n">
         <v>6</v>
       </c>
-      <c r="C78" s="27" t="n">
+      <c r="C80" s="27" t="n">
         <v>10</v>
       </c>
-      <c r="D78" s="27" t="n">
+      <c r="D80" s="27" t="n">
         <v>10</v>
       </c>
-      <c r="E78" s="27" t="n">
+      <c r="E80" s="27" t="n">
         <v>10</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>Gross margin %</t>
-        </is>
-      </c>
-      <c r="B79" s="25" t="n">
-        <v>0.74227032572702</v>
-      </c>
-      <c r="C79" s="25" t="n">
-        <v>0.7413371483484427</v>
-      </c>
-      <c r="D79" s="25" t="n">
-        <v>0.7417480051896446</v>
-      </c>
-      <c r="E79" s="25" t="n">
-        <v>0.7416628553477914</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>Peak cash need before external funding</t>
-        </is>
-      </c>
-      <c r="B80" s="30" t="n">
-        <v>36337.05</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Month of peak cash need</t>
-        </is>
-      </c>
-      <c r="B81" s="31" t="n">
-        <v>7</v>
+          <t>Gross margin %</t>
+        </is>
+      </c>
+      <c r="B81" s="25" t="n">
+        <v>0.74227032572702</v>
+      </c>
+      <c r="C81" s="25" t="n">
+        <v>0.7413371483484427</v>
+      </c>
+      <c r="D81" s="25" t="n">
+        <v>0.7417480051896446</v>
+      </c>
+      <c r="E81" s="25" t="n">
+        <v>0.7416628553477914</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>First month with positive EBITDA</t>
-        </is>
-      </c>
-      <c r="B82" s="31" t="n">
-        <v>2</v>
+          <t>Peak cash need before external funding</t>
+        </is>
+      </c>
+      <c r="B82" s="30" t="n">
+        <v>144704.74</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>First month cumulative result positive</t>
+          <t>Month of peak cash need</t>
         </is>
       </c>
       <c r="B83" s="31" t="n">
-        <v>9</v>
+        <v>31</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Minimum closing cash after funding</t>
-        </is>
-      </c>
-      <c r="B84" s="30" t="n">
-        <v>-18845.15</v>
+          <t>First month with positive EBITDA (may be a blip)</t>
+        </is>
+      </c>
+      <c r="B84" s="31" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Month of minimum closing cash</t>
+          <t>First month of SUSTAINED positive EBITDA (break-even)</t>
         </is>
       </c>
       <c r="B85" s="31" t="n">
-        <v>2</v>
+        <v>31</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Closing cash month 36</t>
-        </is>
-      </c>
-      <c r="B86" s="30" t="n">
-        <v>11350389.66</v>
+          <t>First month cumulative result positive</t>
+        </is>
+      </c>
+      <c r="B86" s="31" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Equity raised in model</t>
+          <t>Minimum closing cash after funding</t>
         </is>
       </c>
       <c r="B87" s="30" t="n">
-        <v>9500000</v>
+        <v>12750</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Grants in model</t>
-        </is>
-      </c>
-      <c r="B88" s="30" t="n">
-        <v>400000</v>
+          <t>Month of minimum closing cash</t>
+        </is>
+      </c>
+      <c r="B88" s="31" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
+          <t>Closing cash month 36</t>
+        </is>
+      </c>
+      <c r="B89" s="30" t="n">
+        <v>3839984.81</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Equity raised in model</t>
+        </is>
+      </c>
+      <c r="B90" s="30" t="n">
+        <v>3500000</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Grants in model</t>
+        </is>
+      </c>
+      <c r="B91" s="30" t="n">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
           <t>Runway at month 36 (months)</t>
         </is>
       </c>
-      <c r="B89" s="32" t="inlineStr">
+      <c r="B92" s="32" t="inlineStr">
         <is>
           <t>cash-generative</t>
         </is>
@@ -4211,17 +4310,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Opening cash (founder capital, month 1)</t>
+          <t>Opening cash (founder capital + director's loan, month 1)</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>10000</v>
+        <v>25000</v>
       </c>
       <c r="D9" s="11" t="n">
-        <v>20000</v>
+        <v>35000</v>
       </c>
       <c r="E9" s="11" t="n">
-        <v>30000</v>
+        <v>50000</v>
       </c>
       <c r="F9" s="12">
         <f>INDEX($C9:$E9,1,$C$4)</f>
@@ -4239,7 +4338,7 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Founder's own contribution; TO VALIDATE with founder.</t>
+          <t>Founder's own contribution incl. a director's loan that bridges month-1 set-up costs until the pre-seed lands; TO VALIDATE with founder. (Revised 8 Sept 2026 from £10k/£20k/£30k, which left cash negative in months 2–5 of every scenario.)</t>
         </is>
       </c>
     </row>
@@ -6348,10 +6447,10 @@
         <v>4</v>
       </c>
       <c r="D68" s="13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E68" s="13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F68" s="14">
         <f>INDEX($C68:$E68,1,$C$4)</f>
@@ -6369,7 +6468,7 @@
       </c>
       <c r="I68" s="4" t="inlineStr">
         <is>
-          <t>Conservative: founder draws nothing until first invoices are paid.</t>
+          <t>Founder draws nothing until the first invoices (month 2) are collected (month 3, one-month lag). Conservative waits one more month. (Revised 8 Sept 2026 from 4/2/1.)</t>
         </is>
       </c>
     </row>
@@ -6497,7 +6596,7 @@
         </is>
       </c>
       <c r="C72" s="13" t="n">
-        <v>19</v>
+        <v>99</v>
       </c>
       <c r="D72" s="13" t="n">
         <v>10</v>
@@ -6519,7 +6618,11 @@
           <t>ASSUMPTION</t>
         </is>
       </c>
-      <c r="I72" s="4" t="inlineStr"/>
+      <c r="I72" s="4" t="inlineStr">
+        <is>
+          <t>Conservative: not hired — a £250k pre-seed cannot carry a second technical salary (cash went negative at month 31 when it was); contractors instead. (Revised 8 Sept 2026 from month 19.)</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
@@ -7092,7 +7195,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Contractors (dev, design, fractional clinical safety officer) — Y1</t>
+          <t>Contractors (dev, design, implementation, fractional clinical safety officer) — Y1</t>
         </is>
       </c>
       <c r="C89" s="11" t="n">
@@ -7128,17 +7231,17 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Contractors (dev, design, fractional clinical safety officer) — Y2</t>
+          <t>Contractors (dev, design, implementation, fractional clinical safety officer) — Y2</t>
         </is>
       </c>
       <c r="C90" s="11" t="n">
         <v>4000</v>
       </c>
       <c r="D90" s="11" t="n">
-        <v>6000</v>
+        <v>10000</v>
       </c>
       <c r="E90" s="11" t="n">
-        <v>6000</v>
+        <v>20000</v>
       </c>
       <c r="F90" s="12">
         <f>INDEX($C90:$E90,1,$C$4)</f>
@@ -7164,17 +7267,17 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Contractors (dev, design, fractional clinical safety officer) — Y3</t>
+          <t>Contractors (dev, design, implementation, fractional clinical safety officer) — Y3</t>
         </is>
       </c>
       <c r="C91" s="11" t="n">
         <v>8000</v>
       </c>
       <c r="D91" s="11" t="n">
-        <v>10000</v>
+        <v>30000</v>
       </c>
       <c r="E91" s="11" t="n">
-        <v>8000</v>
+        <v>45000</v>
       </c>
       <c r="F91" s="12">
         <f>INDEX($C91:$E91,1,$C$4)</f>
@@ -7243,10 +7346,10 @@
         <v>600</v>
       </c>
       <c r="D93" s="11" t="n">
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="E93" s="11" t="n">
-        <v>3000</v>
+        <v>6000</v>
       </c>
       <c r="F93" s="12">
         <f>INDEX($C93:$E93,1,$C$4)</f>
@@ -7279,10 +7382,10 @@
         <v>1500</v>
       </c>
       <c r="D94" s="11" t="n">
-        <v>4000</v>
+        <v>10000</v>
       </c>
       <c r="E94" s="11" t="n">
-        <v>8000</v>
+        <v>20000</v>
       </c>
       <c r="F94" s="12">
         <f>INDEX($C94:$E94,1,$C$4)</f>
@@ -7308,7 +7411,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Marketing (content, events, paid tests) — Y1</t>
+          <t>Marketing (content, events, paid tests, demand generation) — Y1</t>
         </is>
       </c>
       <c r="C95" s="11" t="n">
@@ -7344,17 +7447,17 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Marketing (content, events, paid tests) — Y2</t>
+          <t>Marketing (content, events, paid tests, demand generation) — Y2</t>
         </is>
       </c>
       <c r="C96" s="11" t="n">
         <v>750</v>
       </c>
       <c r="D96" s="11" t="n">
-        <v>2000</v>
+        <v>4000</v>
       </c>
       <c r="E96" s="11" t="n">
-        <v>3000</v>
+        <v>12000</v>
       </c>
       <c r="F96" s="12">
         <f>INDEX($C96:$E96,1,$C$4)</f>
@@ -7380,17 +7483,17 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Marketing (content, events, paid tests) — Y3</t>
+          <t>Marketing (content, events, paid tests, demand generation) — Y3</t>
         </is>
       </c>
       <c r="C97" s="11" t="n">
         <v>2000</v>
       </c>
       <c r="D97" s="11" t="n">
-        <v>5000</v>
+        <v>15000</v>
       </c>
       <c r="E97" s="11" t="n">
-        <v>8000</v>
+        <v>35000</v>
       </c>
       <c r="F97" s="12">
         <f>INDEX($C97:$E97,1,$C$4)</f>
@@ -7570,7 +7673,7 @@
         <v>1000</v>
       </c>
       <c r="E102" s="11" t="n">
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="F102" s="12">
         <f>INDEX($C102:$E102,1,$C$4)</f>
@@ -7603,10 +7706,10 @@
         <v>600</v>
       </c>
       <c r="D103" s="11" t="n">
-        <v>2000</v>
+        <v>4000</v>
       </c>
       <c r="E103" s="11" t="n">
-        <v>3000</v>
+        <v>5000</v>
       </c>
       <c r="F103" s="12">
         <f>INDEX($C103:$E103,1,$C$4)</f>
@@ -7891,10 +7994,10 @@
         <v>400</v>
       </c>
       <c r="D111" s="11" t="n">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="E111" s="11" t="n">
-        <v>1500</v>
+        <v>4000</v>
       </c>
       <c r="F111" s="12">
         <f>INDEX($C111:$E111,1,$C$4)</f>
@@ -7927,10 +8030,10 @@
         <v>800</v>
       </c>
       <c r="D112" s="11" t="n">
-        <v>2500</v>
+        <v>6000</v>
       </c>
       <c r="E112" s="11" t="n">
-        <v>4000</v>
+        <v>10000</v>
       </c>
       <c r="F112" s="12">
         <f>INDEX($C112:$E112,1,$C$4)</f>
@@ -7956,7 +8059,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Operations (co-working, recruitment, misc.) — Y1</t>
+          <t>Operations (co-working, recruitment, in-country field support, misc.) — Y1</t>
         </is>
       </c>
       <c r="C113" s="11" t="n">
@@ -7992,17 +8095,17 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Operations (co-working, recruitment, misc.) — Y2</t>
+          <t>Operations (co-working, recruitment, in-country field support, misc.) — Y2</t>
         </is>
       </c>
       <c r="C114" s="11" t="n">
         <v>250</v>
       </c>
       <c r="D114" s="11" t="n">
-        <v>800</v>
+        <v>1500</v>
       </c>
       <c r="E114" s="11" t="n">
-        <v>1500</v>
+        <v>5000</v>
       </c>
       <c r="F114" s="12">
         <f>INDEX($C114:$E114,1,$C$4)</f>
@@ -8028,17 +8131,17 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Operations (co-working, recruitment, misc.) — Y3</t>
+          <t>Operations (co-working, recruitment, in-country field support, misc.) — Y3</t>
         </is>
       </c>
       <c r="C115" s="11" t="n">
         <v>500</v>
       </c>
       <c r="D115" s="11" t="n">
-        <v>2000</v>
+        <v>8000</v>
       </c>
       <c r="E115" s="11" t="n">
-        <v>4000</v>
+        <v>15000</v>
       </c>
       <c r="F115" s="12">
         <f>INDEX($C115:$E115,1,$C$4)</f>
@@ -8388,8 +8491,8 @@
       <c r="D125" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="E125" s="11" t="n">
-        <v>6000000</v>
+      <c r="E125" s="17" t="n">
+        <v>0</v>
       </c>
       <c r="F125" s="18">
         <f>INDEX($C125:$E125,1,$C$4)</f>
@@ -8407,7 +8510,7 @@
       </c>
       <c r="I125" s="4" t="inlineStr">
         <is>
-          <t>High-growth only, month 32.</t>
+          <t>Not in the 36-month model in any scenario: no scenario needs it for solvency within 36 months, and High-growth reaches EBITDA break-even. Series A (£6m–£12m) is a month 30–42 growth-capital decision — see 09_FUNDING_STRATEGY. Set an amount and month here to test it. (Revised 8 Sept 2026: was £6m at month 32 in High-growth, raised while cash-generative with £4m in the bank.)</t>
         </is>
       </c>
     </row>
@@ -8429,7 +8532,7 @@
         <v>99</v>
       </c>
       <c r="E126" s="13" t="n">
-        <v>32</v>
+        <v>99</v>
       </c>
       <c r="F126" s="14">
         <f>INDEX($C126:$E126,1,$C$4)</f>
@@ -19675,7 +19778,7 @@
     <row r="16">
       <c r="A16" s="22" t="inlineStr">
         <is>
-          <t>Contractors (dev, design, fractional clinical safety officer)</t>
+          <t>Contractors (dev, design, implementation, fractional clinical safety officer)</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr"/>
@@ -20011,7 +20114,7 @@
     <row r="18">
       <c r="A18" s="22" t="inlineStr">
         <is>
-          <t>Marketing (content, events, paid tests)</t>
+          <t>Marketing (content, events, paid tests, demand generation)</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr"/>
@@ -21019,7 +21122,7 @@
     <row r="24">
       <c r="A24" s="22" t="inlineStr">
         <is>
-          <t>Operations (co-working, recruitment, misc.)</t>
+          <t>Operations (co-working, recruitment, in-country field support, misc.)</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr"/>
@@ -30566,7 +30669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ39"/>
+  <dimension ref="A1:AQ40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -35279,661 +35382,813 @@
     <row r="34">
       <c r="A34" s="22" t="inlineStr">
         <is>
+          <t>EBITDA positive from this month to month 36 (1/0) — sustained break-even</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr"/>
+      <c r="C34" s="27">
+        <f>IF(MIN(C32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="D34" s="27">
+        <f>IF(MIN(D32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="E34" s="27">
+        <f>IF(MIN(E32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="F34" s="27">
+        <f>IF(MIN(F32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="G34" s="27">
+        <f>IF(MIN(G32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="H34" s="27">
+        <f>IF(MIN(H32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="I34" s="27">
+        <f>IF(MIN(I32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="J34" s="27">
+        <f>IF(MIN(J32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="K34" s="27">
+        <f>IF(MIN(K32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="L34" s="27">
+        <f>IF(MIN(L32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M34" s="27">
+        <f>IF(MIN(M32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="N34" s="27">
+        <f>IF(MIN(N32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="O34" s="27">
+        <f>IF(MIN(O32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="P34" s="27">
+        <f>IF(MIN(P32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="Q34" s="27">
+        <f>IF(MIN(Q32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="R34" s="27">
+        <f>IF(MIN(R32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="S34" s="27">
+        <f>IF(MIN(S32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="T34" s="27">
+        <f>IF(MIN(T32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="U34" s="27">
+        <f>IF(MIN(U32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="V34" s="27">
+        <f>IF(MIN(V32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="W34" s="27">
+        <f>IF(MIN(W32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="X34" s="27">
+        <f>IF(MIN(X32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="Y34" s="27">
+        <f>IF(MIN(Y32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="Z34" s="27">
+        <f>IF(MIN(Z32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AA34" s="27">
+        <f>IF(MIN(AA32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AB34" s="27">
+        <f>IF(MIN(AB32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AC34" s="27">
+        <f>IF(MIN(AC32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AD34" s="27">
+        <f>IF(MIN(AD32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AE34" s="27">
+        <f>IF(MIN(AE32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AF34" s="27">
+        <f>IF(MIN(AF32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AG34" s="27">
+        <f>IF(MIN(AG32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AH34" s="27">
+        <f>IF(MIN(AH32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AI34" s="27">
+        <f>IF(MIN(AI32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AJ34" s="27">
+        <f>IF(MIN(AJ32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AK34" s="27">
+        <f>IF(MIN(AK32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AL34" s="27">
+        <f>IF(MIN(AL32:AL32)&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="22" t="inlineStr">
+        <is>
           <t>Grant income (other income; TO VALIDATE)</t>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr"/>
-      <c r="C34" s="19">
+      <c r="B35" s="4" t="inlineStr"/>
+      <c r="C35" s="19">
         <f>'Cash flow'!C18</f>
         <v/>
       </c>
-      <c r="D34" s="19">
+      <c r="D35" s="19">
         <f>'Cash flow'!D18</f>
         <v/>
       </c>
-      <c r="E34" s="19">
+      <c r="E35" s="19">
         <f>'Cash flow'!E18</f>
         <v/>
       </c>
-      <c r="F34" s="19">
+      <c r="F35" s="19">
         <f>'Cash flow'!F18</f>
         <v/>
       </c>
-      <c r="G34" s="19">
+      <c r="G35" s="19">
         <f>'Cash flow'!G18</f>
         <v/>
       </c>
-      <c r="H34" s="19">
+      <c r="H35" s="19">
         <f>'Cash flow'!H18</f>
         <v/>
       </c>
-      <c r="I34" s="19">
+      <c r="I35" s="19">
         <f>'Cash flow'!I18</f>
         <v/>
       </c>
-      <c r="J34" s="19">
+      <c r="J35" s="19">
         <f>'Cash flow'!J18</f>
         <v/>
       </c>
-      <c r="K34" s="19">
+      <c r="K35" s="19">
         <f>'Cash flow'!K18</f>
         <v/>
       </c>
-      <c r="L34" s="19">
+      <c r="L35" s="19">
         <f>'Cash flow'!L18</f>
         <v/>
       </c>
-      <c r="M34" s="19">
+      <c r="M35" s="19">
         <f>'Cash flow'!M18</f>
         <v/>
       </c>
-      <c r="N34" s="19">
+      <c r="N35" s="19">
         <f>'Cash flow'!N18</f>
         <v/>
       </c>
-      <c r="O34" s="19">
+      <c r="O35" s="19">
         <f>'Cash flow'!O18</f>
         <v/>
       </c>
-      <c r="P34" s="19">
+      <c r="P35" s="19">
         <f>'Cash flow'!P18</f>
         <v/>
       </c>
-      <c r="Q34" s="19">
+      <c r="Q35" s="19">
         <f>'Cash flow'!Q18</f>
         <v/>
       </c>
-      <c r="R34" s="19">
+      <c r="R35" s="19">
         <f>'Cash flow'!R18</f>
         <v/>
       </c>
-      <c r="S34" s="19">
+      <c r="S35" s="19">
         <f>'Cash flow'!S18</f>
         <v/>
       </c>
-      <c r="T34" s="19">
+      <c r="T35" s="19">
         <f>'Cash flow'!T18</f>
         <v/>
       </c>
-      <c r="U34" s="19">
+      <c r="U35" s="19">
         <f>'Cash flow'!U18</f>
         <v/>
       </c>
-      <c r="V34" s="19">
+      <c r="V35" s="19">
         <f>'Cash flow'!V18</f>
         <v/>
       </c>
-      <c r="W34" s="19">
+      <c r="W35" s="19">
         <f>'Cash flow'!W18</f>
         <v/>
       </c>
-      <c r="X34" s="19">
+      <c r="X35" s="19">
         <f>'Cash flow'!X18</f>
         <v/>
       </c>
-      <c r="Y34" s="19">
+      <c r="Y35" s="19">
         <f>'Cash flow'!Y18</f>
         <v/>
       </c>
-      <c r="Z34" s="19">
+      <c r="Z35" s="19">
         <f>'Cash flow'!Z18</f>
         <v/>
       </c>
-      <c r="AA34" s="19">
+      <c r="AA35" s="19">
         <f>'Cash flow'!AA18</f>
         <v/>
       </c>
-      <c r="AB34" s="19">
+      <c r="AB35" s="19">
         <f>'Cash flow'!AB18</f>
         <v/>
       </c>
-      <c r="AC34" s="19">
+      <c r="AC35" s="19">
         <f>'Cash flow'!AC18</f>
         <v/>
       </c>
-      <c r="AD34" s="19">
+      <c r="AD35" s="19">
         <f>'Cash flow'!AD18</f>
         <v/>
       </c>
-      <c r="AE34" s="19">
+      <c r="AE35" s="19">
         <f>'Cash flow'!AE18</f>
         <v/>
       </c>
-      <c r="AF34" s="19">
+      <c r="AF35" s="19">
         <f>'Cash flow'!AF18</f>
         <v/>
       </c>
-      <c r="AG34" s="19">
+      <c r="AG35" s="19">
         <f>'Cash flow'!AG18</f>
         <v/>
       </c>
-      <c r="AH34" s="19">
+      <c r="AH35" s="19">
         <f>'Cash flow'!AH18</f>
         <v/>
       </c>
-      <c r="AI34" s="19">
+      <c r="AI35" s="19">
         <f>'Cash flow'!AI18</f>
         <v/>
       </c>
-      <c r="AJ34" s="19">
+      <c r="AJ35" s="19">
         <f>'Cash flow'!AJ18</f>
         <v/>
       </c>
-      <c r="AK34" s="19">
+      <c r="AK35" s="19">
         <f>'Cash flow'!AK18</f>
         <v/>
       </c>
-      <c r="AL34" s="19">
+      <c r="AL35" s="19">
         <f>'Cash flow'!AL18</f>
         <v/>
       </c>
-      <c r="AN34" s="19">
-        <f>SUMIF($C$5:$AL$5,AN$5,C34:AL34)</f>
-        <v/>
-      </c>
-      <c r="AO34" s="19">
-        <f>SUMIF($C$5:$AL$5,AO$5,C34:AL34)</f>
-        <v/>
-      </c>
-      <c r="AP34" s="19">
-        <f>SUMIF($C$5:$AL$5,AP$5,C34:AL34)</f>
-        <v/>
-      </c>
-      <c r="AQ34" s="19">
-        <f>SUM(C34:AL34)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="7" t="inlineStr">
+      <c r="AN35" s="19">
+        <f>SUMIF($C$5:$AL$5,AN$5,C35:AL35)</f>
+        <v/>
+      </c>
+      <c r="AO35" s="19">
+        <f>SUMIF($C$5:$AL$5,AO$5,C35:AL35)</f>
+        <v/>
+      </c>
+      <c r="AP35" s="19">
+        <f>SUMIF($C$5:$AL$5,AP$5,C35:AL35)</f>
+        <v/>
+      </c>
+      <c r="AQ35" s="19">
+        <f>SUM(C35:AL35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
         <is>
           <t>NET RESULT BEFORE TAX</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr"/>
-      <c r="C35" s="26">
-        <f>'P&amp;L'!C32+'P&amp;L'!C34</f>
-        <v/>
-      </c>
-      <c r="D35" s="26">
-        <f>'P&amp;L'!D32+'P&amp;L'!D34</f>
-        <v/>
-      </c>
-      <c r="E35" s="26">
-        <f>'P&amp;L'!E32+'P&amp;L'!E34</f>
-        <v/>
-      </c>
-      <c r="F35" s="26">
-        <f>'P&amp;L'!F32+'P&amp;L'!F34</f>
-        <v/>
-      </c>
-      <c r="G35" s="26">
-        <f>'P&amp;L'!G32+'P&amp;L'!G34</f>
-        <v/>
-      </c>
-      <c r="H35" s="26">
-        <f>'P&amp;L'!H32+'P&amp;L'!H34</f>
-        <v/>
-      </c>
-      <c r="I35" s="26">
-        <f>'P&amp;L'!I32+'P&amp;L'!I34</f>
-        <v/>
-      </c>
-      <c r="J35" s="26">
-        <f>'P&amp;L'!J32+'P&amp;L'!J34</f>
-        <v/>
-      </c>
-      <c r="K35" s="26">
-        <f>'P&amp;L'!K32+'P&amp;L'!K34</f>
-        <v/>
-      </c>
-      <c r="L35" s="26">
-        <f>'P&amp;L'!L32+'P&amp;L'!L34</f>
-        <v/>
-      </c>
-      <c r="M35" s="26">
-        <f>'P&amp;L'!M32+'P&amp;L'!M34</f>
-        <v/>
-      </c>
-      <c r="N35" s="26">
-        <f>'P&amp;L'!N32+'P&amp;L'!N34</f>
-        <v/>
-      </c>
-      <c r="O35" s="26">
-        <f>'P&amp;L'!O32+'P&amp;L'!O34</f>
-        <v/>
-      </c>
-      <c r="P35" s="26">
-        <f>'P&amp;L'!P32+'P&amp;L'!P34</f>
-        <v/>
-      </c>
-      <c r="Q35" s="26">
-        <f>'P&amp;L'!Q32+'P&amp;L'!Q34</f>
-        <v/>
-      </c>
-      <c r="R35" s="26">
-        <f>'P&amp;L'!R32+'P&amp;L'!R34</f>
-        <v/>
-      </c>
-      <c r="S35" s="26">
-        <f>'P&amp;L'!S32+'P&amp;L'!S34</f>
-        <v/>
-      </c>
-      <c r="T35" s="26">
-        <f>'P&amp;L'!T32+'P&amp;L'!T34</f>
-        <v/>
-      </c>
-      <c r="U35" s="26">
-        <f>'P&amp;L'!U32+'P&amp;L'!U34</f>
-        <v/>
-      </c>
-      <c r="V35" s="26">
-        <f>'P&amp;L'!V32+'P&amp;L'!V34</f>
-        <v/>
-      </c>
-      <c r="W35" s="26">
-        <f>'P&amp;L'!W32+'P&amp;L'!W34</f>
-        <v/>
-      </c>
-      <c r="X35" s="26">
-        <f>'P&amp;L'!X32+'P&amp;L'!X34</f>
-        <v/>
-      </c>
-      <c r="Y35" s="26">
-        <f>'P&amp;L'!Y32+'P&amp;L'!Y34</f>
-        <v/>
-      </c>
-      <c r="Z35" s="26">
-        <f>'P&amp;L'!Z32+'P&amp;L'!Z34</f>
-        <v/>
-      </c>
-      <c r="AA35" s="26">
-        <f>'P&amp;L'!AA32+'P&amp;L'!AA34</f>
-        <v/>
-      </c>
-      <c r="AB35" s="26">
-        <f>'P&amp;L'!AB32+'P&amp;L'!AB34</f>
-        <v/>
-      </c>
-      <c r="AC35" s="26">
-        <f>'P&amp;L'!AC32+'P&amp;L'!AC34</f>
-        <v/>
-      </c>
-      <c r="AD35" s="26">
-        <f>'P&amp;L'!AD32+'P&amp;L'!AD34</f>
-        <v/>
-      </c>
-      <c r="AE35" s="26">
-        <f>'P&amp;L'!AE32+'P&amp;L'!AE34</f>
-        <v/>
-      </c>
-      <c r="AF35" s="26">
-        <f>'P&amp;L'!AF32+'P&amp;L'!AF34</f>
-        <v/>
-      </c>
-      <c r="AG35" s="26">
-        <f>'P&amp;L'!AG32+'P&amp;L'!AG34</f>
-        <v/>
-      </c>
-      <c r="AH35" s="26">
-        <f>'P&amp;L'!AH32+'P&amp;L'!AH34</f>
-        <v/>
-      </c>
-      <c r="AI35" s="26">
-        <f>'P&amp;L'!AI32+'P&amp;L'!AI34</f>
-        <v/>
-      </c>
-      <c r="AJ35" s="26">
-        <f>'P&amp;L'!AJ32+'P&amp;L'!AJ34</f>
-        <v/>
-      </c>
-      <c r="AK35" s="26">
-        <f>'P&amp;L'!AK32+'P&amp;L'!AK34</f>
-        <v/>
-      </c>
-      <c r="AL35" s="26">
-        <f>'P&amp;L'!AL32+'P&amp;L'!AL34</f>
-        <v/>
-      </c>
-      <c r="AN35" s="26">
-        <f>SUMIF($C$5:$AL$5,AN$5,C35:AL35)</f>
-        <v/>
-      </c>
-      <c r="AO35" s="26">
-        <f>SUMIF($C$5:$AL$5,AO$5,C35:AL35)</f>
-        <v/>
-      </c>
-      <c r="AP35" s="26">
-        <f>SUMIF($C$5:$AL$5,AP$5,C35:AL35)</f>
-        <v/>
-      </c>
-      <c r="AQ35" s="26">
-        <f>SUM(C35:AL35)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="22" t="inlineStr">
-        <is>
-          <t>Cumulative net result</t>
-        </is>
-      </c>
       <c r="B36" s="4" t="inlineStr"/>
-      <c r="C36" s="19">
-        <f>'P&amp;L'!C35</f>
-        <v/>
-      </c>
-      <c r="D36" s="19">
-        <f>'P&amp;L'!C36+'P&amp;L'!D35</f>
-        <v/>
-      </c>
-      <c r="E36" s="19">
-        <f>'P&amp;L'!D36+'P&amp;L'!E35</f>
-        <v/>
-      </c>
-      <c r="F36" s="19">
-        <f>'P&amp;L'!E36+'P&amp;L'!F35</f>
-        <v/>
-      </c>
-      <c r="G36" s="19">
-        <f>'P&amp;L'!F36+'P&amp;L'!G35</f>
-        <v/>
-      </c>
-      <c r="H36" s="19">
-        <f>'P&amp;L'!G36+'P&amp;L'!H35</f>
-        <v/>
-      </c>
-      <c r="I36" s="19">
-        <f>'P&amp;L'!H36+'P&amp;L'!I35</f>
-        <v/>
-      </c>
-      <c r="J36" s="19">
-        <f>'P&amp;L'!I36+'P&amp;L'!J35</f>
-        <v/>
-      </c>
-      <c r="K36" s="19">
-        <f>'P&amp;L'!J36+'P&amp;L'!K35</f>
-        <v/>
-      </c>
-      <c r="L36" s="19">
-        <f>'P&amp;L'!K36+'P&amp;L'!L35</f>
-        <v/>
-      </c>
-      <c r="M36" s="19">
-        <f>'P&amp;L'!L36+'P&amp;L'!M35</f>
-        <v/>
-      </c>
-      <c r="N36" s="19">
-        <f>'P&amp;L'!M36+'P&amp;L'!N35</f>
-        <v/>
-      </c>
-      <c r="O36" s="19">
-        <f>'P&amp;L'!N36+'P&amp;L'!O35</f>
-        <v/>
-      </c>
-      <c r="P36" s="19">
-        <f>'P&amp;L'!O36+'P&amp;L'!P35</f>
-        <v/>
-      </c>
-      <c r="Q36" s="19">
-        <f>'P&amp;L'!P36+'P&amp;L'!Q35</f>
-        <v/>
-      </c>
-      <c r="R36" s="19">
-        <f>'P&amp;L'!Q36+'P&amp;L'!R35</f>
-        <v/>
-      </c>
-      <c r="S36" s="19">
-        <f>'P&amp;L'!R36+'P&amp;L'!S35</f>
-        <v/>
-      </c>
-      <c r="T36" s="19">
-        <f>'P&amp;L'!S36+'P&amp;L'!T35</f>
-        <v/>
-      </c>
-      <c r="U36" s="19">
-        <f>'P&amp;L'!T36+'P&amp;L'!U35</f>
-        <v/>
-      </c>
-      <c r="V36" s="19">
-        <f>'P&amp;L'!U36+'P&amp;L'!V35</f>
-        <v/>
-      </c>
-      <c r="W36" s="19">
-        <f>'P&amp;L'!V36+'P&amp;L'!W35</f>
-        <v/>
-      </c>
-      <c r="X36" s="19">
-        <f>'P&amp;L'!W36+'P&amp;L'!X35</f>
-        <v/>
-      </c>
-      <c r="Y36" s="19">
-        <f>'P&amp;L'!X36+'P&amp;L'!Y35</f>
-        <v/>
-      </c>
-      <c r="Z36" s="19">
-        <f>'P&amp;L'!Y36+'P&amp;L'!Z35</f>
-        <v/>
-      </c>
-      <c r="AA36" s="19">
-        <f>'P&amp;L'!Z36+'P&amp;L'!AA35</f>
-        <v/>
-      </c>
-      <c r="AB36" s="19">
-        <f>'P&amp;L'!AA36+'P&amp;L'!AB35</f>
-        <v/>
-      </c>
-      <c r="AC36" s="19">
-        <f>'P&amp;L'!AB36+'P&amp;L'!AC35</f>
-        <v/>
-      </c>
-      <c r="AD36" s="19">
-        <f>'P&amp;L'!AC36+'P&amp;L'!AD35</f>
-        <v/>
-      </c>
-      <c r="AE36" s="19">
-        <f>'P&amp;L'!AD36+'P&amp;L'!AE35</f>
-        <v/>
-      </c>
-      <c r="AF36" s="19">
-        <f>'P&amp;L'!AE36+'P&amp;L'!AF35</f>
-        <v/>
-      </c>
-      <c r="AG36" s="19">
-        <f>'P&amp;L'!AF36+'P&amp;L'!AG35</f>
-        <v/>
-      </c>
-      <c r="AH36" s="19">
-        <f>'P&amp;L'!AG36+'P&amp;L'!AH35</f>
-        <v/>
-      </c>
-      <c r="AI36" s="19">
-        <f>'P&amp;L'!AH36+'P&amp;L'!AI35</f>
-        <v/>
-      </c>
-      <c r="AJ36" s="19">
-        <f>'P&amp;L'!AI36+'P&amp;L'!AJ35</f>
-        <v/>
-      </c>
-      <c r="AK36" s="19">
-        <f>'P&amp;L'!AJ36+'P&amp;L'!AK35</f>
-        <v/>
-      </c>
-      <c r="AL36" s="19">
-        <f>'P&amp;L'!AK36+'P&amp;L'!AL35</f>
-        <v/>
-      </c>
-      <c r="AN36" s="19">
-        <f>INDEX(C36:AL36,1,12)</f>
-        <v/>
-      </c>
-      <c r="AO36" s="19">
-        <f>INDEX(C36:AL36,1,24)</f>
-        <v/>
-      </c>
-      <c r="AP36" s="19">
-        <f>INDEX(C36:AL36,1,36)</f>
-        <v/>
-      </c>
-      <c r="AQ36" s="19">
-        <f>INDEX(C36:AL36,1,36)</f>
+      <c r="C36" s="26">
+        <f>'P&amp;L'!C32+'P&amp;L'!C35</f>
+        <v/>
+      </c>
+      <c r="D36" s="26">
+        <f>'P&amp;L'!D32+'P&amp;L'!D35</f>
+        <v/>
+      </c>
+      <c r="E36" s="26">
+        <f>'P&amp;L'!E32+'P&amp;L'!E35</f>
+        <v/>
+      </c>
+      <c r="F36" s="26">
+        <f>'P&amp;L'!F32+'P&amp;L'!F35</f>
+        <v/>
+      </c>
+      <c r="G36" s="26">
+        <f>'P&amp;L'!G32+'P&amp;L'!G35</f>
+        <v/>
+      </c>
+      <c r="H36" s="26">
+        <f>'P&amp;L'!H32+'P&amp;L'!H35</f>
+        <v/>
+      </c>
+      <c r="I36" s="26">
+        <f>'P&amp;L'!I32+'P&amp;L'!I35</f>
+        <v/>
+      </c>
+      <c r="J36" s="26">
+        <f>'P&amp;L'!J32+'P&amp;L'!J35</f>
+        <v/>
+      </c>
+      <c r="K36" s="26">
+        <f>'P&amp;L'!K32+'P&amp;L'!K35</f>
+        <v/>
+      </c>
+      <c r="L36" s="26">
+        <f>'P&amp;L'!L32+'P&amp;L'!L35</f>
+        <v/>
+      </c>
+      <c r="M36" s="26">
+        <f>'P&amp;L'!M32+'P&amp;L'!M35</f>
+        <v/>
+      </c>
+      <c r="N36" s="26">
+        <f>'P&amp;L'!N32+'P&amp;L'!N35</f>
+        <v/>
+      </c>
+      <c r="O36" s="26">
+        <f>'P&amp;L'!O32+'P&amp;L'!O35</f>
+        <v/>
+      </c>
+      <c r="P36" s="26">
+        <f>'P&amp;L'!P32+'P&amp;L'!P35</f>
+        <v/>
+      </c>
+      <c r="Q36" s="26">
+        <f>'P&amp;L'!Q32+'P&amp;L'!Q35</f>
+        <v/>
+      </c>
+      <c r="R36" s="26">
+        <f>'P&amp;L'!R32+'P&amp;L'!R35</f>
+        <v/>
+      </c>
+      <c r="S36" s="26">
+        <f>'P&amp;L'!S32+'P&amp;L'!S35</f>
+        <v/>
+      </c>
+      <c r="T36" s="26">
+        <f>'P&amp;L'!T32+'P&amp;L'!T35</f>
+        <v/>
+      </c>
+      <c r="U36" s="26">
+        <f>'P&amp;L'!U32+'P&amp;L'!U35</f>
+        <v/>
+      </c>
+      <c r="V36" s="26">
+        <f>'P&amp;L'!V32+'P&amp;L'!V35</f>
+        <v/>
+      </c>
+      <c r="W36" s="26">
+        <f>'P&amp;L'!W32+'P&amp;L'!W35</f>
+        <v/>
+      </c>
+      <c r="X36" s="26">
+        <f>'P&amp;L'!X32+'P&amp;L'!X35</f>
+        <v/>
+      </c>
+      <c r="Y36" s="26">
+        <f>'P&amp;L'!Y32+'P&amp;L'!Y35</f>
+        <v/>
+      </c>
+      <c r="Z36" s="26">
+        <f>'P&amp;L'!Z32+'P&amp;L'!Z35</f>
+        <v/>
+      </c>
+      <c r="AA36" s="26">
+        <f>'P&amp;L'!AA32+'P&amp;L'!AA35</f>
+        <v/>
+      </c>
+      <c r="AB36" s="26">
+        <f>'P&amp;L'!AB32+'P&amp;L'!AB35</f>
+        <v/>
+      </c>
+      <c r="AC36" s="26">
+        <f>'P&amp;L'!AC32+'P&amp;L'!AC35</f>
+        <v/>
+      </c>
+      <c r="AD36" s="26">
+        <f>'P&amp;L'!AD32+'P&amp;L'!AD35</f>
+        <v/>
+      </c>
+      <c r="AE36" s="26">
+        <f>'P&amp;L'!AE32+'P&amp;L'!AE35</f>
+        <v/>
+      </c>
+      <c r="AF36" s="26">
+        <f>'P&amp;L'!AF32+'P&amp;L'!AF35</f>
+        <v/>
+      </c>
+      <c r="AG36" s="26">
+        <f>'P&amp;L'!AG32+'P&amp;L'!AG35</f>
+        <v/>
+      </c>
+      <c r="AH36" s="26">
+        <f>'P&amp;L'!AH32+'P&amp;L'!AH35</f>
+        <v/>
+      </c>
+      <c r="AI36" s="26">
+        <f>'P&amp;L'!AI32+'P&amp;L'!AI35</f>
+        <v/>
+      </c>
+      <c r="AJ36" s="26">
+        <f>'P&amp;L'!AJ32+'P&amp;L'!AJ35</f>
+        <v/>
+      </c>
+      <c r="AK36" s="26">
+        <f>'P&amp;L'!AK32+'P&amp;L'!AK35</f>
+        <v/>
+      </c>
+      <c r="AL36" s="26">
+        <f>'P&amp;L'!AL32+'P&amp;L'!AL35</f>
+        <v/>
+      </c>
+      <c r="AN36" s="26">
+        <f>SUMIF($C$5:$AL$5,AN$5,C36:AL36)</f>
+        <v/>
+      </c>
+      <c r="AO36" s="26">
+        <f>SUMIF($C$5:$AL$5,AO$5,C36:AL36)</f>
+        <v/>
+      </c>
+      <c r="AP36" s="26">
+        <f>SUMIF($C$5:$AL$5,AP$5,C36:AL36)</f>
+        <v/>
+      </c>
+      <c r="AQ36" s="26">
+        <f>SUM(C36:AL36)</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="22" t="inlineStr">
         <is>
+          <t>Cumulative net result</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr"/>
+      <c r="C37" s="19">
+        <f>'P&amp;L'!C36</f>
+        <v/>
+      </c>
+      <c r="D37" s="19">
+        <f>'P&amp;L'!C37+'P&amp;L'!D36</f>
+        <v/>
+      </c>
+      <c r="E37" s="19">
+        <f>'P&amp;L'!D37+'P&amp;L'!E36</f>
+        <v/>
+      </c>
+      <c r="F37" s="19">
+        <f>'P&amp;L'!E37+'P&amp;L'!F36</f>
+        <v/>
+      </c>
+      <c r="G37" s="19">
+        <f>'P&amp;L'!F37+'P&amp;L'!G36</f>
+        <v/>
+      </c>
+      <c r="H37" s="19">
+        <f>'P&amp;L'!G37+'P&amp;L'!H36</f>
+        <v/>
+      </c>
+      <c r="I37" s="19">
+        <f>'P&amp;L'!H37+'P&amp;L'!I36</f>
+        <v/>
+      </c>
+      <c r="J37" s="19">
+        <f>'P&amp;L'!I37+'P&amp;L'!J36</f>
+        <v/>
+      </c>
+      <c r="K37" s="19">
+        <f>'P&amp;L'!J37+'P&amp;L'!K36</f>
+        <v/>
+      </c>
+      <c r="L37" s="19">
+        <f>'P&amp;L'!K37+'P&amp;L'!L36</f>
+        <v/>
+      </c>
+      <c r="M37" s="19">
+        <f>'P&amp;L'!L37+'P&amp;L'!M36</f>
+        <v/>
+      </c>
+      <c r="N37" s="19">
+        <f>'P&amp;L'!M37+'P&amp;L'!N36</f>
+        <v/>
+      </c>
+      <c r="O37" s="19">
+        <f>'P&amp;L'!N37+'P&amp;L'!O36</f>
+        <v/>
+      </c>
+      <c r="P37" s="19">
+        <f>'P&amp;L'!O37+'P&amp;L'!P36</f>
+        <v/>
+      </c>
+      <c r="Q37" s="19">
+        <f>'P&amp;L'!P37+'P&amp;L'!Q36</f>
+        <v/>
+      </c>
+      <c r="R37" s="19">
+        <f>'P&amp;L'!Q37+'P&amp;L'!R36</f>
+        <v/>
+      </c>
+      <c r="S37" s="19">
+        <f>'P&amp;L'!R37+'P&amp;L'!S36</f>
+        <v/>
+      </c>
+      <c r="T37" s="19">
+        <f>'P&amp;L'!S37+'P&amp;L'!T36</f>
+        <v/>
+      </c>
+      <c r="U37" s="19">
+        <f>'P&amp;L'!T37+'P&amp;L'!U36</f>
+        <v/>
+      </c>
+      <c r="V37" s="19">
+        <f>'P&amp;L'!U37+'P&amp;L'!V36</f>
+        <v/>
+      </c>
+      <c r="W37" s="19">
+        <f>'P&amp;L'!V37+'P&amp;L'!W36</f>
+        <v/>
+      </c>
+      <c r="X37" s="19">
+        <f>'P&amp;L'!W37+'P&amp;L'!X36</f>
+        <v/>
+      </c>
+      <c r="Y37" s="19">
+        <f>'P&amp;L'!X37+'P&amp;L'!Y36</f>
+        <v/>
+      </c>
+      <c r="Z37" s="19">
+        <f>'P&amp;L'!Y37+'P&amp;L'!Z36</f>
+        <v/>
+      </c>
+      <c r="AA37" s="19">
+        <f>'P&amp;L'!Z37+'P&amp;L'!AA36</f>
+        <v/>
+      </c>
+      <c r="AB37" s="19">
+        <f>'P&amp;L'!AA37+'P&amp;L'!AB36</f>
+        <v/>
+      </c>
+      <c r="AC37" s="19">
+        <f>'P&amp;L'!AB37+'P&amp;L'!AC36</f>
+        <v/>
+      </c>
+      <c r="AD37" s="19">
+        <f>'P&amp;L'!AC37+'P&amp;L'!AD36</f>
+        <v/>
+      </c>
+      <c r="AE37" s="19">
+        <f>'P&amp;L'!AD37+'P&amp;L'!AE36</f>
+        <v/>
+      </c>
+      <c r="AF37" s="19">
+        <f>'P&amp;L'!AE37+'P&amp;L'!AF36</f>
+        <v/>
+      </c>
+      <c r="AG37" s="19">
+        <f>'P&amp;L'!AF37+'P&amp;L'!AG36</f>
+        <v/>
+      </c>
+      <c r="AH37" s="19">
+        <f>'P&amp;L'!AG37+'P&amp;L'!AH36</f>
+        <v/>
+      </c>
+      <c r="AI37" s="19">
+        <f>'P&amp;L'!AH37+'P&amp;L'!AI36</f>
+        <v/>
+      </c>
+      <c r="AJ37" s="19">
+        <f>'P&amp;L'!AI37+'P&amp;L'!AJ36</f>
+        <v/>
+      </c>
+      <c r="AK37" s="19">
+        <f>'P&amp;L'!AJ37+'P&amp;L'!AK36</f>
+        <v/>
+      </c>
+      <c r="AL37" s="19">
+        <f>'P&amp;L'!AK37+'P&amp;L'!AL36</f>
+        <v/>
+      </c>
+      <c r="AN37" s="19">
+        <f>INDEX(C37:AL37,1,12)</f>
+        <v/>
+      </c>
+      <c r="AO37" s="19">
+        <f>INDEX(C37:AL37,1,24)</f>
+        <v/>
+      </c>
+      <c r="AP37" s="19">
+        <f>INDEX(C37:AL37,1,36)</f>
+        <v/>
+      </c>
+      <c r="AQ37" s="19">
+        <f>INDEX(C37:AL37,1,36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="22" t="inlineStr">
+        <is>
           <t>Cumulative result positive (1/0)</t>
         </is>
       </c>
-      <c r="B37" s="4" t="inlineStr"/>
-      <c r="C37" s="27">
-        <f>IF('P&amp;L'!C36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="D37" s="27">
-        <f>IF('P&amp;L'!D36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="E37" s="27">
-        <f>IF('P&amp;L'!E36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="F37" s="27">
-        <f>IF('P&amp;L'!F36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="G37" s="27">
-        <f>IF('P&amp;L'!G36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="H37" s="27">
-        <f>IF('P&amp;L'!H36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="I37" s="27">
-        <f>IF('P&amp;L'!I36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="J37" s="27">
-        <f>IF('P&amp;L'!J36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="K37" s="27">
-        <f>IF('P&amp;L'!K36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="L37" s="27">
-        <f>IF('P&amp;L'!L36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="M37" s="27">
-        <f>IF('P&amp;L'!M36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="N37" s="27">
-        <f>IF('P&amp;L'!N36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="O37" s="27">
-        <f>IF('P&amp;L'!O36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="P37" s="27">
-        <f>IF('P&amp;L'!P36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="Q37" s="27">
-        <f>IF('P&amp;L'!Q36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="R37" s="27">
-        <f>IF('P&amp;L'!R36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="S37" s="27">
-        <f>IF('P&amp;L'!S36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="T37" s="27">
-        <f>IF('P&amp;L'!T36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="U37" s="27">
-        <f>IF('P&amp;L'!U36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="V37" s="27">
-        <f>IF('P&amp;L'!V36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="W37" s="27">
-        <f>IF('P&amp;L'!W36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="X37" s="27">
-        <f>IF('P&amp;L'!X36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="Y37" s="27">
-        <f>IF('P&amp;L'!Y36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="Z37" s="27">
-        <f>IF('P&amp;L'!Z36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="AA37" s="27">
-        <f>IF('P&amp;L'!AA36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="AB37" s="27">
-        <f>IF('P&amp;L'!AB36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="AC37" s="27">
-        <f>IF('P&amp;L'!AC36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="AD37" s="27">
-        <f>IF('P&amp;L'!AD36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="AE37" s="27">
-        <f>IF('P&amp;L'!AE36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="AF37" s="27">
-        <f>IF('P&amp;L'!AF36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="AG37" s="27">
-        <f>IF('P&amp;L'!AG36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="AH37" s="27">
-        <f>IF('P&amp;L'!AH36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="AI37" s="27">
-        <f>IF('P&amp;L'!AI36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="AJ37" s="27">
-        <f>IF('P&amp;L'!AJ36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="AK37" s="27">
-        <f>IF('P&amp;L'!AK36&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="AL37" s="27">
-        <f>IF('P&amp;L'!AL36&gt;0,1,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
+      <c r="B38" s="4" t="inlineStr"/>
+      <c r="C38" s="27">
+        <f>IF('P&amp;L'!C37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="D38" s="27">
+        <f>IF('P&amp;L'!D37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="E38" s="27">
+        <f>IF('P&amp;L'!E37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="F38" s="27">
+        <f>IF('P&amp;L'!F37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="G38" s="27">
+        <f>IF('P&amp;L'!G37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="H38" s="27">
+        <f>IF('P&amp;L'!H37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="I38" s="27">
+        <f>IF('P&amp;L'!I37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="J38" s="27">
+        <f>IF('P&amp;L'!J37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="K38" s="27">
+        <f>IF('P&amp;L'!K37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="L38" s="27">
+        <f>IF('P&amp;L'!L37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M38" s="27">
+        <f>IF('P&amp;L'!M37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="N38" s="27">
+        <f>IF('P&amp;L'!N37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="O38" s="27">
+        <f>IF('P&amp;L'!O37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="P38" s="27">
+        <f>IF('P&amp;L'!P37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="Q38" s="27">
+        <f>IF('P&amp;L'!Q37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="R38" s="27">
+        <f>IF('P&amp;L'!R37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="S38" s="27">
+        <f>IF('P&amp;L'!S37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="T38" s="27">
+        <f>IF('P&amp;L'!T37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="U38" s="27">
+        <f>IF('P&amp;L'!U37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="V38" s="27">
+        <f>IF('P&amp;L'!V37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="W38" s="27">
+        <f>IF('P&amp;L'!W37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="X38" s="27">
+        <f>IF('P&amp;L'!X37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="Y38" s="27">
+        <f>IF('P&amp;L'!Y37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="Z38" s="27">
+        <f>IF('P&amp;L'!Z37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AA38" s="27">
+        <f>IF('P&amp;L'!AA37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AB38" s="27">
+        <f>IF('P&amp;L'!AB37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AC38" s="27">
+        <f>IF('P&amp;L'!AC37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AD38" s="27">
+        <f>IF('P&amp;L'!AD37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AE38" s="27">
+        <f>IF('P&amp;L'!AE37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AF38" s="27">
+        <f>IF('P&amp;L'!AF37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AG38" s="27">
+        <f>IF('P&amp;L'!AG37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AH38" s="27">
+        <f>IF('P&amp;L'!AH37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AI38" s="27">
+        <f>IF('P&amp;L'!AI37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AJ38" s="27">
+        <f>IF('P&amp;L'!AJ37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AK38" s="27">
+        <f>IF('P&amp;L'!AK37&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AL38" s="27">
+        <f>IF('P&amp;L'!AL37&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>No depreciation, interest, corporation tax or VAT modelled (loss-making; R&amp;D tax relief is an unmodelled upside, TO VALIDATE).</t>
         </is>
@@ -39831,7 +40086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="78" customWidth="1" min="1" max="1"/>
@@ -39916,7 +40171,7 @@
         </is>
       </c>
       <c r="B9" s="31">
-        <f>IFERROR(MATCH(1,'P&amp;L'!$C$37:$AL$37,0),"Not reached in 36 months")</f>
+        <f>IFERROR(MATCH(1,'P&amp;L'!$C$38:$AL$38,0),"Not reached in 36 months")</f>
         <v/>
       </c>
     </row>
@@ -40030,185 +40285,196 @@
         <v/>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>First month of SUSTAINED positive EBITDA (stays positive to month 36)</t>
+        </is>
+      </c>
+      <c r="B20" s="31">
+        <f>IFERROR(MATCH(1,'P&amp;L'!$C$34:$AL$34,0),"Not reached in 36 months")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Funding rounds in the active scenario (PROPOSED; every round is conditional on the milestones in 09_FUNDING_STRATEGY.md)</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>Round</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>Amount (GBP)</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr">
+      <c r="E23" s="7" t="inlineStr">
         <is>
           <t>Cumulative cash before this round (model)</t>
         </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Pre-seed (SEIS/EIS)</t>
-        </is>
-      </c>
-      <c r="B23">
-        <f>Assumptions!$F$122</f>
-        <v/>
-      </c>
-      <c r="C23">
-        <f>IF(Assumptions!$F$122&lt;=36,TEXT(DATE(2027,Assumptions!$F$122,1),"mmm yyyy"),"not in model")</f>
-        <v/>
-      </c>
-      <c r="D23" s="19">
-        <f>Assumptions!$F$121</f>
-        <v/>
-      </c>
-      <c r="E23" s="19">
-        <f>IF(Assumptions!$F$122&lt;=36,INDEX('Cash flow'!$C$27:$AL$27,1,Assumptions!$F$122),"—")</f>
-        <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Seed</t>
+          <t>Pre-seed (SEIS/EIS)</t>
         </is>
       </c>
       <c r="B24">
-        <f>Assumptions!$F$124</f>
+        <f>Assumptions!$F$122</f>
         <v/>
       </c>
       <c r="C24">
-        <f>IF(Assumptions!$F$124&lt;=36,TEXT(DATE(2027,Assumptions!$F$124,1),"mmm yyyy"),"not in model")</f>
+        <f>IF(Assumptions!$F$122&lt;=36,TEXT(DATE(2027,Assumptions!$F$122,1),"mmm yyyy"),"not in model")</f>
         <v/>
       </c>
       <c r="D24" s="19">
-        <f>Assumptions!$F$123</f>
+        <f>Assumptions!$F$121</f>
         <v/>
       </c>
       <c r="E24" s="19">
-        <f>IF(Assumptions!$F$124&lt;=36,INDEX('Cash flow'!$C$27:$AL$27,1,Assumptions!$F$124),"—")</f>
+        <f>IF(Assumptions!$F$122&lt;=36,INDEX('Cash flow'!$C$27:$AL$27,1,Assumptions!$F$122),"—")</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Series A</t>
+          <t>Seed</t>
         </is>
       </c>
       <c r="B25">
-        <f>Assumptions!$F$126</f>
+        <f>Assumptions!$F$124</f>
         <v/>
       </c>
       <c r="C25">
-        <f>IF(Assumptions!$F$126&lt;=36,TEXT(DATE(2027,Assumptions!$F$126,1),"mmm yyyy"),"not in model")</f>
+        <f>IF(Assumptions!$F$124&lt;=36,TEXT(DATE(2027,Assumptions!$F$124,1),"mmm yyyy"),"not in model")</f>
         <v/>
       </c>
       <c r="D25" s="19">
-        <f>Assumptions!$F$125</f>
+        <f>Assumptions!$F$123</f>
         <v/>
       </c>
       <c r="E25" s="19">
-        <f>IF(Assumptions!$F$126&lt;=36,INDEX('Cash flow'!$C$27:$AL$27,1,Assumptions!$F$126),"—")</f>
+        <f>IF(Assumptions!$F$124&lt;=36,INDEX('Cash flow'!$C$27:$AL$27,1,Assumptions!$F$124),"—")</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Grant 1</t>
+          <t>Series A</t>
         </is>
       </c>
       <c r="B26">
-        <f>Assumptions!$F$128</f>
+        <f>Assumptions!$F$126</f>
         <v/>
       </c>
       <c r="C26">
-        <f>IF(Assumptions!$F$128&lt;=36,TEXT(DATE(2027,Assumptions!$F$128,1),"mmm yyyy"),"not in model")</f>
+        <f>IF(Assumptions!$F$126&lt;=36,TEXT(DATE(2027,Assumptions!$F$126,1),"mmm yyyy"),"not in model")</f>
         <v/>
       </c>
       <c r="D26" s="19">
-        <f>Assumptions!$F$127</f>
+        <f>Assumptions!$F$125</f>
         <v/>
       </c>
       <c r="E26" s="19">
-        <f>IF(Assumptions!$F$128&lt;=36,INDEX('Cash flow'!$C$27:$AL$27,1,Assumptions!$F$128),"—")</f>
+        <f>IF(Assumptions!$F$126&lt;=36,INDEX('Cash flow'!$C$27:$AL$27,1,Assumptions!$F$126),"—")</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>Grant 1</t>
+        </is>
+      </c>
+      <c r="B27">
+        <f>Assumptions!$F$128</f>
+        <v/>
+      </c>
+      <c r="C27">
+        <f>IF(Assumptions!$F$128&lt;=36,TEXT(DATE(2027,Assumptions!$F$128,1),"mmm yyyy"),"not in model")</f>
+        <v/>
+      </c>
+      <c r="D27" s="19">
+        <f>Assumptions!$F$127</f>
+        <v/>
+      </c>
+      <c r="E27" s="19">
+        <f>IF(Assumptions!$F$128&lt;=36,INDEX('Cash flow'!$C$27:$AL$27,1,Assumptions!$F$128),"—")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>Grant 2</t>
         </is>
       </c>
-      <c r="B27">
+      <c r="B28">
         <f>Assumptions!$F$130</f>
         <v/>
       </c>
-      <c r="C27">
+      <c r="C28">
         <f>IF(Assumptions!$F$130&lt;=36,TEXT(DATE(2027,Assumptions!$F$130,1),"mmm yyyy"),"not in model")</f>
         <v/>
       </c>
-      <c r="D27" s="19">
+      <c r="D28" s="19">
         <f>Assumptions!$F$129</f>
         <v/>
       </c>
-      <c r="E27" s="19">
+      <c r="E28" s="19">
         <f>IF(Assumptions!$F$130&lt;=36,INDEX('Cash flow'!$C$27:$AL$27,1,Assumptions!$F$130),"—")</f>
         <v/>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>Reading this sheet</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>• Peak cash need is the external money required to keep cash ≥ 0 with no equity or grants — the number to raise (plus a buffer of 20–30%).</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>• Break-even = first month EBITDA &gt; 0 (before grant income). Cumulative break-even is when losses to date are recovered.</t>
+          <t>• Peak cash need is the external money required to keep cash ≥ 0 with no equity or grants — the number to raise (plus a buffer of 20–30%).</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>• If the funded-through check shows SHORTFALL, the scenario's rounds are too small or too late for its cost base.</t>
+          <t>• Break-even = first month EBITDA &gt; 0 (before grant income) — this can be a pre-salary blip in months 2–4; use the SUSTAINED figure (row 20) as the real break-even. Cumulative break-even is when losses to date are recovered.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>• If the funded-through check shows SHORTFALL, the scenario's rounds are too small or too late for its cost base.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>• Grants are recognised when received; they are competitive and none is secured (TO VALIDATE).</t>
         </is>

</xml_diff>